<commit_message>
Update music stats and options
</commit_message>
<xml_diff>
--- a/musicscores/Openingnotes.xlsx
+++ b/musicscores/Openingnotes.xlsx
@@ -16,11 +16,12 @@
     <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="145621"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1844" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1861" uniqueCount="757">
   <si>
     <t xml:space="preserve">e </t>
   </si>
@@ -2255,13 +2256,49 @@
   </si>
   <si>
     <t>PDF PAGES at 13 pt +</t>
+  </si>
+  <si>
+    <t>@.02/page</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Royalty</t>
+  </si>
+  <si>
+    <t>Published volume</t>
+  </si>
+  <si>
+    <t>Back Cover</t>
+  </si>
+  <si>
+    <t>LAC Descr</t>
+  </si>
+  <si>
+    <t>Press Rel.</t>
+  </si>
+  <si>
+    <t>ISBN</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>PDF Size</t>
+  </si>
+  <si>
+    <t>Cover</t>
+  </si>
+  <si>
+    <t>Amazon</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="7">
+  <numFmts count="9">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
@@ -2269,6 +2306,8 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="170" formatCode="_-[$$-1009]* #,##0.00_-;\-[$$-1009]* #,##0.00_-;_-[$$-1009]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="yyyy/mm/dd;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -2420,7 +2459,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2456,6 +2495,10 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -2789,11 +2832,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="240245248"/>
-        <c:axId val="141319488"/>
+        <c:axId val="177232384"/>
+        <c:axId val="191074240"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="240245248"/>
+        <c:axId val="177232384"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2802,7 +2845,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="141319488"/>
+        <c:crossAx val="191074240"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2810,7 +2853,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="141319488"/>
+        <c:axId val="191074240"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2821,7 +2864,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="240245248"/>
+        <c:crossAx val="177232384"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3165,11 +3208,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="241598464"/>
-        <c:axId val="231268928"/>
+        <c:axId val="177103872"/>
+        <c:axId val="191075392"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="241598464"/>
+        <c:axId val="177103872"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3178,7 +3221,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="231268928"/>
+        <c:crossAx val="191075392"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3186,7 +3229,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="231268928"/>
+        <c:axId val="191075392"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3197,7 +3240,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="241598464"/>
+        <c:crossAx val="177103872"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3437,11 +3480,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="241600000"/>
-        <c:axId val="231271232"/>
+        <c:axId val="177105408"/>
+        <c:axId val="191077696"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="241600000"/>
+        <c:axId val="177105408"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3450,7 +3493,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="231271232"/>
+        <c:crossAx val="191077696"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3458,7 +3501,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="231271232"/>
+        <c:axId val="191077696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3469,7 +3512,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="241600000"/>
+        <c:crossAx val="177105408"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3866,11 +3909,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="215813120"/>
-        <c:axId val="231274688"/>
+        <c:axId val="178267136"/>
+        <c:axId val="177007424"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="215813120"/>
+        <c:axId val="178267136"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3879,7 +3922,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="231274688"/>
+        <c:crossAx val="177007424"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3887,7 +3930,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="231274688"/>
+        <c:axId val="177007424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3898,7 +3941,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="215813120"/>
+        <c:crossAx val="178267136"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4363,11 +4406,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="241601024"/>
-        <c:axId val="231275840"/>
+        <c:axId val="178267648"/>
+        <c:axId val="177009152"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="241601024"/>
+        <c:axId val="178267648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4376,7 +4419,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="231275840"/>
+        <c:crossAx val="177009152"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4384,7 +4427,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="231275840"/>
+        <c:axId val="177009152"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4395,7 +4438,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="241601024"/>
+        <c:crossAx val="178267648"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4688,12 +4731,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="241829888"/>
-        <c:axId val="241797952"/>
+        <c:axId val="178269696"/>
+        <c:axId val="177012032"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="241829888"/>
+        <c:axId val="178269696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4702,7 +4745,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="241797952"/>
+        <c:crossAx val="177012032"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4710,7 +4753,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="241797952"/>
+        <c:axId val="177012032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4721,7 +4764,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="241829888"/>
+        <c:crossAx val="178269696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5783,7 +5826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T47"/>
+  <dimension ref="A1:T65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -5791,7 +5834,9 @@
     <col min="5" max="5" width="9.85546875" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.140625" customWidth="1"/>
     <col min="16" max="16" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.28515625" customWidth="1"/>
@@ -7188,6 +7233,15 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F26" s="8"/>
+      <c r="I26" s="7" t="s">
+        <v>745</v>
+      </c>
+      <c r="J26" t="s">
+        <v>746</v>
+      </c>
+      <c r="K26" t="s">
+        <v>747</v>
+      </c>
       <c r="L26" t="s">
         <v>139</v>
       </c>
@@ -7212,6 +7266,16 @@
       <c r="F27" t="s">
         <v>744</v>
       </c>
+      <c r="I27">
+        <f>0.02</f>
+        <v>0.02</v>
+      </c>
+      <c r="J27">
+        <v>8.9590000000000003E-2</v>
+      </c>
+      <c r="K27">
+        <v>0.4</v>
+      </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
@@ -7238,6 +7302,18 @@
       </c>
       <c r="G28" s="20"/>
       <c r="H28" s="20"/>
+      <c r="I28" s="35">
+        <f>$I$27*F28</f>
+        <v>8.48</v>
+      </c>
+      <c r="J28" s="35">
+        <f>$J$27*F28</f>
+        <v>37.986159999999998</v>
+      </c>
+      <c r="K28" s="35">
+        <f>J28*$K$27</f>
+        <v>15.194464</v>
+      </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
@@ -7256,7 +7332,7 @@
         <v>40</v>
       </c>
       <c r="E29">
-        <f t="shared" ref="E29" si="10">E6</f>
+        <f t="shared" ref="E29:E45" si="10">E6</f>
         <v>1213</v>
       </c>
       <c r="F29" s="20">
@@ -7264,6 +7340,18 @@
       </c>
       <c r="G29" s="20"/>
       <c r="H29" s="20"/>
+      <c r="I29" s="35">
+        <f t="shared" ref="I29:I45" si="11">$I$27*F29</f>
+        <v>7.12</v>
+      </c>
+      <c r="J29" s="35">
+        <f t="shared" ref="J29:J45" si="12">$J$27*F29</f>
+        <v>31.89404</v>
+      </c>
+      <c r="K29" s="35">
+        <f t="shared" ref="K29:K46" si="13">J29*$K$27</f>
+        <v>12.757616000000001</v>
+      </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
@@ -7282,7 +7370,7 @@
         <v>27</v>
       </c>
       <c r="E30">
-        <f t="shared" ref="E30" si="11">E7</f>
+        <f t="shared" si="10"/>
         <v>859</v>
       </c>
       <c r="F30" s="20">
@@ -7290,9 +7378,18 @@
       </c>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
-      <c r="I30" s="20"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="20"/>
+      <c r="I30" s="35">
+        <f t="shared" si="11"/>
+        <v>4.84</v>
+      </c>
+      <c r="J30" s="35">
+        <f t="shared" si="12"/>
+        <v>21.680780000000002</v>
+      </c>
+      <c r="K30" s="35">
+        <f t="shared" si="13"/>
+        <v>8.6723120000000016</v>
+      </c>
       <c r="L30" s="20"/>
       <c r="M30" s="20"/>
       <c r="N30" t="s">
@@ -7305,7 +7402,7 @@
         <v>341</v>
       </c>
       <c r="Q30" s="1">
-        <f>P30/O30</f>
+        <f t="shared" ref="Q30:Q35" si="14">P30/O30</f>
         <v>9.1298527443105751E-2</v>
       </c>
     </row>
@@ -7326,7 +7423,7 @@
         <v>36</v>
       </c>
       <c r="E31">
-        <f t="shared" ref="E31" si="12">E8</f>
+        <f t="shared" si="10"/>
         <v>1288</v>
       </c>
       <c r="F31" s="20">
@@ -7334,9 +7431,18 @@
       </c>
       <c r="G31" s="20"/>
       <c r="H31" s="20"/>
-      <c r="I31" s="20"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
+      <c r="I31" s="35">
+        <f t="shared" si="11"/>
+        <v>6.9</v>
+      </c>
+      <c r="J31" s="35">
+        <f t="shared" si="12"/>
+        <v>30.908550000000002</v>
+      </c>
+      <c r="K31" s="35">
+        <f t="shared" si="13"/>
+        <v>12.363420000000001</v>
+      </c>
       <c r="L31" s="20"/>
       <c r="M31" s="20"/>
       <c r="N31" t="s">
@@ -7349,7 +7455,7 @@
         <v>1297</v>
       </c>
       <c r="Q31" s="1">
-        <f t="shared" ref="Q31:Q35" si="13">P31/O31</f>
+        <f t="shared" si="14"/>
         <v>0.29211711711711713</v>
       </c>
     </row>
@@ -7370,7 +7476,7 @@
         <v>34</v>
       </c>
       <c r="E32">
-        <f t="shared" ref="E32" si="14">E9</f>
+        <f t="shared" si="10"/>
         <v>959</v>
       </c>
       <c r="F32" s="20">
@@ -7383,9 +7489,18 @@
         <f>L32</f>
         <v>1660</v>
       </c>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
+      <c r="I32" s="35">
+        <f t="shared" si="11"/>
+        <v>5.86</v>
+      </c>
+      <c r="J32" s="35">
+        <f t="shared" si="12"/>
+        <v>26.249870000000001</v>
+      </c>
+      <c r="K32" s="35">
+        <f t="shared" si="13"/>
+        <v>10.499948000000002</v>
+      </c>
       <c r="L32" s="20">
         <f>SUM(F28:F32)</f>
         <v>1660</v>
@@ -7401,7 +7516,7 @@
         <v>1239</v>
       </c>
       <c r="Q32" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>9.5860735009671183E-2</v>
       </c>
     </row>
@@ -7422,7 +7537,7 @@
         <v>45</v>
       </c>
       <c r="E33">
-        <f t="shared" ref="E33" si="15">E10</f>
+        <f t="shared" si="10"/>
         <v>1276</v>
       </c>
       <c r="F33" s="20">
@@ -7430,9 +7545,18 @@
       </c>
       <c r="G33" s="20"/>
       <c r="H33" s="20"/>
-      <c r="I33" s="20"/>
-      <c r="J33" s="20"/>
-      <c r="K33" s="20"/>
+      <c r="I33" s="35">
+        <f t="shared" si="11"/>
+        <v>7.86</v>
+      </c>
+      <c r="J33" s="35">
+        <f t="shared" si="12"/>
+        <v>35.208870000000005</v>
+      </c>
+      <c r="K33" s="35">
+        <f t="shared" si="13"/>
+        <v>14.083548000000002</v>
+      </c>
       <c r="L33" s="20"/>
       <c r="M33" s="20"/>
       <c r="N33" t="s">
@@ -7445,7 +7569,7 @@
         <v>255</v>
       </c>
       <c r="Q33" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.12160228898426323</v>
       </c>
     </row>
@@ -7466,7 +7590,7 @@
         <v>55</v>
       </c>
       <c r="E34">
-        <f t="shared" ref="E34" si="16">E11</f>
+        <f t="shared" si="10"/>
         <v>1505</v>
       </c>
       <c r="F34" s="20">
@@ -7474,9 +7598,18 @@
       </c>
       <c r="G34" s="20"/>
       <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
-      <c r="J34" s="20"/>
-      <c r="K34" s="20"/>
+      <c r="I34" s="35">
+        <f t="shared" si="11"/>
+        <v>9.34</v>
+      </c>
+      <c r="J34" s="35">
+        <f t="shared" si="12"/>
+        <v>41.838529999999999</v>
+      </c>
+      <c r="K34" s="35">
+        <f t="shared" si="13"/>
+        <v>16.735412</v>
+      </c>
       <c r="L34" s="20"/>
       <c r="M34" s="20"/>
       <c r="O34">
@@ -7488,7 +7621,7 @@
         <v>3132</v>
       </c>
       <c r="Q34" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.13501745915420096</v>
       </c>
     </row>
@@ -7509,7 +7642,7 @@
         <v>47</v>
       </c>
       <c r="E35">
-        <f t="shared" ref="E35" si="17">E12</f>
+        <f t="shared" si="10"/>
         <v>1536</v>
       </c>
       <c r="F35" s="20">
@@ -7517,9 +7650,18 @@
       </c>
       <c r="G35" s="20"/>
       <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
-      <c r="J35" s="20"/>
-      <c r="K35" s="20"/>
+      <c r="I35" s="35">
+        <f t="shared" si="11"/>
+        <v>9.7000000000000011</v>
+      </c>
+      <c r="J35" s="35">
+        <f t="shared" si="12"/>
+        <v>43.451149999999998</v>
+      </c>
+      <c r="K35" s="35">
+        <f t="shared" si="13"/>
+        <v>17.380459999999999</v>
+      </c>
       <c r="L35" s="20">
         <f>SUM(F33:F35)</f>
         <v>1345</v>
@@ -7537,7 +7679,7 @@
         <v>2791</v>
       </c>
       <c r="Q35" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>0.14340766622135442</v>
       </c>
     </row>
@@ -7558,7 +7700,7 @@
         <v>66</v>
       </c>
       <c r="E36">
-        <f t="shared" ref="E36" si="18">E13</f>
+        <f t="shared" si="10"/>
         <v>1291</v>
       </c>
       <c r="F36" s="20">
@@ -7566,9 +7708,18 @@
       </c>
       <c r="G36" s="20"/>
       <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
+      <c r="I36" s="35">
+        <f t="shared" si="11"/>
+        <v>7.54</v>
+      </c>
+      <c r="J36" s="35">
+        <f t="shared" si="12"/>
+        <v>33.77543</v>
+      </c>
+      <c r="K36" s="35">
+        <f t="shared" si="13"/>
+        <v>13.510172000000001</v>
+      </c>
       <c r="L36" s="20"/>
       <c r="M36" s="20"/>
     </row>
@@ -7589,7 +7740,7 @@
         <v>52</v>
       </c>
       <c r="E37">
-        <f t="shared" ref="E37" si="19">E14</f>
+        <f t="shared" si="10"/>
         <v>1364</v>
       </c>
       <c r="F37" s="20">
@@ -7597,9 +7748,18 @@
       </c>
       <c r="G37" s="20"/>
       <c r="H37" s="20"/>
-      <c r="I37" s="20"/>
-      <c r="J37" s="20"/>
-      <c r="K37" s="20"/>
+      <c r="I37" s="35">
+        <f t="shared" si="11"/>
+        <v>8.52</v>
+      </c>
+      <c r="J37" s="35">
+        <f t="shared" si="12"/>
+        <v>38.16534</v>
+      </c>
+      <c r="K37" s="35">
+        <f t="shared" si="13"/>
+        <v>15.266136000000001</v>
+      </c>
       <c r="L37" s="20"/>
       <c r="M37" s="20"/>
       <c r="N37" t="s">
@@ -7629,7 +7789,7 @@
         <v>48</v>
       </c>
       <c r="E38">
-        <f t="shared" ref="E38" si="20">E15</f>
+        <f t="shared" si="10"/>
         <v>1273</v>
       </c>
       <c r="F38" s="20">
@@ -7637,6 +7797,18 @@
       </c>
       <c r="G38" s="20"/>
       <c r="H38" s="20"/>
+      <c r="I38" s="35">
+        <f t="shared" si="11"/>
+        <v>7.78</v>
+      </c>
+      <c r="J38" s="35">
+        <f t="shared" si="12"/>
+        <v>34.85051</v>
+      </c>
+      <c r="K38" s="35">
+        <f t="shared" si="13"/>
+        <v>13.940204000000001</v>
+      </c>
       <c r="N38" t="s">
         <v>732</v>
       </c>
@@ -7664,7 +7836,7 @@
         <v>67</v>
       </c>
       <c r="E39">
-        <f t="shared" ref="E39" si="21">E16</f>
+        <f t="shared" si="10"/>
         <v>1050</v>
       </c>
       <c r="F39" s="20">
@@ -7677,9 +7849,18 @@
         <f>L35+L39</f>
         <v>2864</v>
       </c>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
+      <c r="I39" s="35">
+        <f t="shared" si="11"/>
+        <v>6.54</v>
+      </c>
+      <c r="J39" s="35">
+        <f t="shared" si="12"/>
+        <v>29.295930000000002</v>
+      </c>
+      <c r="K39" s="35">
+        <f t="shared" si="13"/>
+        <v>11.718372000000002</v>
+      </c>
       <c r="L39" s="20">
         <f>SUM(F36:F39)</f>
         <v>1519</v>
@@ -7703,7 +7884,7 @@
         <v>150</v>
       </c>
       <c r="E40">
-        <f t="shared" ref="E40" si="22">E17</f>
+        <f t="shared" si="10"/>
         <v>2527</v>
       </c>
       <c r="F40" s="20">
@@ -7711,9 +7892,18 @@
       </c>
       <c r="G40" s="20"/>
       <c r="H40" s="20"/>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20"/>
-      <c r="K40" s="20"/>
+      <c r="I40" s="35">
+        <f t="shared" si="11"/>
+        <v>11.700000000000001</v>
+      </c>
+      <c r="J40" s="35">
+        <f t="shared" si="12"/>
+        <v>52.410150000000002</v>
+      </c>
+      <c r="K40" s="35">
+        <f t="shared" si="13"/>
+        <v>20.964060000000003</v>
+      </c>
       <c r="L40" s="20"/>
       <c r="M40" s="20"/>
       <c r="N40" t="s">
@@ -7750,7 +7940,7 @@
         <v>31</v>
       </c>
       <c r="E41">
-        <f t="shared" ref="E41" si="23">E18</f>
+        <f t="shared" si="10"/>
         <v>915</v>
       </c>
       <c r="F41" s="20">
@@ -7758,9 +7948,18 @@
       </c>
       <c r="G41" s="20"/>
       <c r="H41" s="20"/>
-      <c r="I41" s="20"/>
-      <c r="J41" s="20"/>
-      <c r="K41" s="20"/>
+      <c r="I41" s="35">
+        <f t="shared" si="11"/>
+        <v>4</v>
+      </c>
+      <c r="J41" s="35">
+        <f t="shared" si="12"/>
+        <v>17.917999999999999</v>
+      </c>
+      <c r="K41" s="35">
+        <f t="shared" si="13"/>
+        <v>7.1672000000000002</v>
+      </c>
       <c r="L41" s="20"/>
       <c r="M41" s="20"/>
       <c r="N41" t="s">
@@ -7797,7 +7996,7 @@
         <v>42</v>
       </c>
       <c r="E42" s="14">
-        <f t="shared" ref="E42" si="24">E19</f>
+        <f t="shared" si="10"/>
         <v>1070</v>
       </c>
       <c r="F42" s="34">
@@ -7805,9 +8004,18 @@
       </c>
       <c r="G42" s="20"/>
       <c r="H42" s="20"/>
-      <c r="I42" s="20"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
+      <c r="I42" s="37">
+        <f t="shared" si="11"/>
+        <v>5.58</v>
+      </c>
+      <c r="J42" s="37">
+        <f t="shared" si="12"/>
+        <v>24.995609999999999</v>
+      </c>
+      <c r="K42" s="37">
+        <f t="shared" si="13"/>
+        <v>9.9982439999999997</v>
+      </c>
       <c r="L42" s="20">
         <f>SUM(F40:F42)</f>
         <v>1064</v>
@@ -7847,11 +8055,23 @@
         <v>39</v>
       </c>
       <c r="E43">
-        <f t="shared" ref="E43" si="25">E20</f>
+        <f t="shared" si="10"/>
         <v>745</v>
       </c>
       <c r="F43" s="20">
         <v>226</v>
+      </c>
+      <c r="I43" s="35">
+        <f t="shared" si="11"/>
+        <v>4.5200000000000005</v>
+      </c>
+      <c r="J43" s="35">
+        <f t="shared" si="12"/>
+        <v>20.247340000000001</v>
+      </c>
+      <c r="K43" s="35">
+        <f t="shared" si="13"/>
+        <v>8.0989360000000001</v>
       </c>
       <c r="N43" s="20" t="s">
         <v>116</v>
@@ -7887,7 +8107,7 @@
         <v>35</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44" si="26">E21</f>
+        <f t="shared" si="10"/>
         <v>1042</v>
       </c>
       <c r="F44" s="20">
@@ -7895,9 +8115,18 @@
       </c>
       <c r="G44" s="20"/>
       <c r="H44" s="20"/>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20"/>
-      <c r="K44" s="20"/>
+      <c r="I44" s="35">
+        <f t="shared" si="11"/>
+        <v>6.38</v>
+      </c>
+      <c r="J44" s="35">
+        <f t="shared" si="12"/>
+        <v>28.57921</v>
+      </c>
+      <c r="K44" s="35">
+        <f t="shared" si="13"/>
+        <v>11.431684000000001</v>
+      </c>
       <c r="L44" s="20"/>
       <c r="M44" s="20"/>
     </row>
@@ -7918,7 +8147,7 @@
         <v>65</v>
       </c>
       <c r="E45">
-        <f t="shared" ref="E45" si="27">E22</f>
+        <f t="shared" si="10"/>
         <v>1750</v>
       </c>
       <c r="F45" s="20">
@@ -7931,9 +8160,18 @@
         <f>L42+L45</f>
         <v>2111</v>
       </c>
-      <c r="I45" s="20"/>
-      <c r="J45" s="20"/>
-      <c r="K45" s="20"/>
+      <c r="I45" s="35">
+        <f t="shared" si="11"/>
+        <v>10.040000000000001</v>
+      </c>
+      <c r="J45" s="35">
+        <f t="shared" si="12"/>
+        <v>44.974180000000004</v>
+      </c>
+      <c r="K45" s="35">
+        <f t="shared" si="13"/>
+        <v>17.989672000000002</v>
+      </c>
       <c r="L45" s="20">
         <f>SUM(F43:F45)</f>
         <v>1047</v>
@@ -7952,7 +8190,7 @@
         <v>28</v>
       </c>
       <c r="R45" s="1">
-        <f t="shared" ref="R45:R47" si="28">Q45/P45</f>
+        <f>Q45/P45</f>
         <v>7.8431372549019607E-2</v>
       </c>
     </row>
@@ -7967,8 +8205,14 @@
         <v>6635</v>
       </c>
       <c r="I46" s="33"/>
-      <c r="J46" s="33"/>
-      <c r="K46" s="33"/>
+      <c r="J46" s="36">
+        <f>SUM(J28:J45)</f>
+        <v>594.42965000000004</v>
+      </c>
+      <c r="K46" s="33">
+        <f t="shared" si="13"/>
+        <v>237.77186000000003</v>
+      </c>
       <c r="L46" s="33">
         <f>SUM(G46:H46)</f>
         <v>6635</v>
@@ -7987,11 +8231,41 @@
         <v>19</v>
       </c>
       <c r="R46" s="1">
-        <f t="shared" si="28"/>
+        <f>Q46/P46</f>
         <v>6.7857142857142852E-2</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B47" t="s">
+        <v>748</v>
+      </c>
+      <c r="D47" t="s">
+        <v>77</v>
+      </c>
+      <c r="E47" t="s">
+        <v>78</v>
+      </c>
+      <c r="F47" t="s">
+        <v>754</v>
+      </c>
+      <c r="G47" t="s">
+        <v>752</v>
+      </c>
+      <c r="H47" t="s">
+        <v>750</v>
+      </c>
+      <c r="I47" t="s">
+        <v>749</v>
+      </c>
+      <c r="J47" t="s">
+        <v>751</v>
+      </c>
+      <c r="K47" t="s">
+        <v>755</v>
+      </c>
+      <c r="L47" t="s">
+        <v>756</v>
+      </c>
       <c r="N47" t="s">
         <v>126</v>
       </c>
@@ -8005,9 +8279,273 @@
         <v>18</v>
       </c>
       <c r="R47" s="1">
-        <f t="shared" si="28"/>
+        <f>Q47/P47</f>
         <v>4.4444444444444446E-2</v>
       </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>1</v>
+      </c>
+      <c r="C48" t="str">
+        <f t="shared" ref="C48:F49" si="15">C42</f>
+        <v>Job</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="15"/>
+        <v>42</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="15"/>
+        <v>1070</v>
+      </c>
+      <c r="F48">
+        <f t="shared" si="15"/>
+        <v>279</v>
+      </c>
+      <c r="G48" t="s">
+        <v>753</v>
+      </c>
+      <c r="H48" s="38">
+        <v>46143</v>
+      </c>
+      <c r="I48" s="38">
+        <v>46023</v>
+      </c>
+      <c r="J48" s="38">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <f>B48+1</f>
+        <v>2</v>
+      </c>
+      <c r="C49" t="str">
+        <f>C40</f>
+        <v>Psalms</v>
+      </c>
+      <c r="D49">
+        <f>D40</f>
+        <v>150</v>
+      </c>
+      <c r="E49">
+        <f>E40</f>
+        <v>2527</v>
+      </c>
+      <c r="F49">
+        <f>F40</f>
+        <v>585</v>
+      </c>
+      <c r="G49" t="s">
+        <v>753</v>
+      </c>
+      <c r="H49" s="38">
+        <v>46143</v>
+      </c>
+      <c r="I49" s="38">
+        <f>H49+1</f>
+        <v>46144</v>
+      </c>
+      <c r="J49" s="38">
+        <f>I49+1</f>
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <f t="shared" ref="B50:B65" si="16">B49+1</f>
+        <v>3</v>
+      </c>
+      <c r="C50" t="str">
+        <f>C43</f>
+        <v>The Five Scrolls</v>
+      </c>
+      <c r="D50">
+        <f>D43</f>
+        <v>39</v>
+      </c>
+      <c r="E50">
+        <f>E43</f>
+        <v>745</v>
+      </c>
+      <c r="F50">
+        <f>F43</f>
+        <v>226</v>
+      </c>
+      <c r="G50" t="s">
+        <v>753</v>
+      </c>
+      <c r="H50" s="38">
+        <v>46143</v>
+      </c>
+      <c r="I50" s="38">
+        <f>H50+1</f>
+        <v>46144</v>
+      </c>
+      <c r="J50" s="38">
+        <f>I50+1</f>
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <f t="shared" si="16"/>
+        <v>4</v>
+      </c>
+      <c r="C51" t="str">
+        <f>C32</f>
+        <v>Deuteronomy</v>
+      </c>
+      <c r="D51">
+        <f>D32</f>
+        <v>34</v>
+      </c>
+      <c r="E51">
+        <f>E32</f>
+        <v>959</v>
+      </c>
+      <c r="F51">
+        <f>F32</f>
+        <v>293</v>
+      </c>
+      <c r="G51" t="s">
+        <v>753</v>
+      </c>
+      <c r="H51" s="38">
+        <v>46143</v>
+      </c>
+      <c r="I51" s="38">
+        <f t="shared" ref="I49:J51" si="17">H51+1</f>
+        <v>46144</v>
+      </c>
+      <c r="J51" s="38">
+        <f t="shared" si="17"/>
+        <v>46145</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <f t="shared" si="16"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <f t="shared" si="16"/>
+        <v>6</v>
+      </c>
+      <c r="H53" s="38"/>
+      <c r="I53" s="38"/>
+      <c r="J53" s="38"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B54">
+        <f t="shared" si="16"/>
+        <v>7</v>
+      </c>
+      <c r="H54" s="38"/>
+      <c r="I54" s="38"/>
+      <c r="J54" s="38"/>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B55">
+        <f t="shared" si="16"/>
+        <v>8</v>
+      </c>
+      <c r="H55" s="38"/>
+      <c r="I55" s="38"/>
+      <c r="J55" s="38"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <f t="shared" si="16"/>
+        <v>9</v>
+      </c>
+      <c r="H56" s="38"/>
+      <c r="I56" s="38"/>
+      <c r="J56" s="38"/>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <f t="shared" si="16"/>
+        <v>10</v>
+      </c>
+      <c r="H57" s="38"/>
+      <c r="I57" s="38"/>
+      <c r="J57" s="38"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <f t="shared" si="16"/>
+        <v>11</v>
+      </c>
+      <c r="H58" s="38"/>
+      <c r="I58" s="38"/>
+      <c r="J58" s="38"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <f t="shared" si="16"/>
+        <v>12</v>
+      </c>
+      <c r="H59" s="38"/>
+      <c r="I59" s="38"/>
+      <c r="J59" s="38"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B60">
+        <f t="shared" si="16"/>
+        <v>13</v>
+      </c>
+      <c r="H60" s="38"/>
+      <c r="I60" s="38"/>
+      <c r="J60" s="38"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <f t="shared" si="16"/>
+        <v>14</v>
+      </c>
+      <c r="H61" s="38"/>
+      <c r="I61" s="38"/>
+      <c r="J61" s="38"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <f t="shared" si="16"/>
+        <v>15</v>
+      </c>
+      <c r="H62" s="38"/>
+      <c r="I62" s="38"/>
+      <c r="J62" s="38"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <f t="shared" si="16"/>
+        <v>16</v>
+      </c>
+      <c r="H63" s="38"/>
+      <c r="I63" s="38"/>
+      <c r="J63" s="38"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B64">
+        <f t="shared" si="16"/>
+        <v>17</v>
+      </c>
+      <c r="H64" s="38"/>
+      <c r="I64" s="38"/>
+      <c r="J64" s="38"/>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <f t="shared" si="16"/>
+        <v>18</v>
+      </c>
+      <c r="H65" s="38"/>
+      <c r="I65" s="38"/>
+      <c r="J65" s="38"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -33186,11 +33724,11 @@
         <v>66</v>
       </c>
       <c r="F17">
-        <f t="shared" ref="F17:G17" si="5">F16-F3-F6-F9-F11-F13</f>
+        <f>F16-F3-F6-F9-F11-F13</f>
         <v>24</v>
       </c>
       <c r="G17">
-        <f t="shared" si="5"/>
+        <f>G16-G3-G6-G9-G11-G13</f>
         <v>13</v>
       </c>
     </row>
@@ -33200,11 +33738,11 @@
         <v>2.6117926394934706E-2</v>
       </c>
       <c r="F18" s="1">
-        <f t="shared" ref="F18:G18" si="6">F17/F16</f>
+        <f>F17/F16</f>
         <v>2.6229508196721311E-2</v>
       </c>
       <c r="G18" s="1">
-        <f t="shared" si="6"/>
+        <f>G17/G16</f>
         <v>1.3026052104208416E-2</v>
       </c>
     </row>
@@ -33442,7 +33980,7 @@
         <v>1</v>
       </c>
       <c r="AM38">
-        <f t="shared" ref="AM38:AM43" si="7">SUM(B38:AL38)</f>
+        <f t="shared" ref="AM38:AM43" si="5">SUM(B38:AL38)</f>
         <v>63</v>
       </c>
     </row>
@@ -33562,7 +34100,7 @@
         <v>1</v>
       </c>
       <c r="AM39">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>96</v>
       </c>
     </row>
@@ -33682,7 +34220,7 @@
         <v>5</v>
       </c>
       <c r="AM40">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>246</v>
       </c>
     </row>
@@ -33802,7 +34340,7 @@
         <v>2</v>
       </c>
       <c r="AM41">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>71</v>
       </c>
     </row>
@@ -33922,7 +34460,7 @@
         <v>20</v>
       </c>
       <c r="AM42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>685</v>
       </c>
     </row>
@@ -34042,7 +34580,7 @@
         <v>21</v>
       </c>
       <c r="AM43">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>583</v>
       </c>
     </row>
@@ -34055,123 +34593,123 @@
         <v>78</v>
       </c>
       <c r="C46">
-        <f t="shared" ref="C46:AF46" si="8">SUM(C38:C45)</f>
+        <f t="shared" ref="C46:AF46" si="6">SUM(C38:C45)</f>
         <v>81</v>
       </c>
       <c r="D46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>87</v>
       </c>
       <c r="E46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>140</v>
       </c>
       <c r="F46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>140</v>
       </c>
       <c r="G46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>65</v>
       </c>
       <c r="H46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>16</v>
       </c>
       <c r="I46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>19</v>
       </c>
       <c r="J46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>30</v>
       </c>
       <c r="K46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>45</v>
       </c>
       <c r="L46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>46</v>
       </c>
       <c r="M46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>226</v>
       </c>
       <c r="N46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>207</v>
       </c>
       <c r="O46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>103</v>
       </c>
       <c r="P46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>32</v>
       </c>
       <c r="Q46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>10</v>
       </c>
       <c r="R46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>26</v>
       </c>
       <c r="S46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="T46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
       <c r="U46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>17</v>
       </c>
       <c r="V46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>12</v>
       </c>
       <c r="W46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>12</v>
       </c>
       <c r="X46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>8</v>
       </c>
       <c r="Y46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>8</v>
       </c>
       <c r="Z46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>34</v>
       </c>
       <c r="AA46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="AB46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>19</v>
       </c>
       <c r="AC46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>3</v>
       </c>
       <c r="AD46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>26</v>
       </c>
       <c r="AE46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>66</v>
       </c>
       <c r="AF46">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>14</v>
       </c>
       <c r="AH46">
@@ -34318,277 +34856,277 @@
     </row>
     <row r="48" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B48">
-        <f t="shared" ref="B48:AF48" si="9">B46+B47</f>
+        <f t="shared" ref="B48:AF48" si="7">B46+B47</f>
         <v>1533</v>
       </c>
       <c r="C48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>1213</v>
       </c>
       <c r="D48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>859</v>
       </c>
       <c r="E48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>1289</v>
       </c>
       <c r="F48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>959</v>
       </c>
       <c r="G48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>658</v>
       </c>
       <c r="H48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>618</v>
       </c>
       <c r="I48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>810</v>
       </c>
       <c r="J48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>695</v>
       </c>
       <c r="K48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>817</v>
       </c>
       <c r="L48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>719</v>
       </c>
       <c r="M48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>1291</v>
       </c>
       <c r="N48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>1364</v>
       </c>
       <c r="O48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>1273</v>
       </c>
       <c r="P48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>197</v>
       </c>
       <c r="Q48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>73</v>
       </c>
       <c r="R48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>146</v>
       </c>
       <c r="S48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>21</v>
       </c>
       <c r="T48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>48</v>
       </c>
       <c r="U48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>105</v>
       </c>
       <c r="V48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>47</v>
       </c>
       <c r="W48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>56</v>
       </c>
       <c r="X48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>53</v>
       </c>
       <c r="Y48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>38</v>
       </c>
       <c r="Z48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>211</v>
       </c>
       <c r="AA48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>55</v>
       </c>
       <c r="AB48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>117</v>
       </c>
       <c r="AC48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>85</v>
       </c>
       <c r="AD48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>154</v>
       </c>
       <c r="AE48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>222</v>
       </c>
       <c r="AF48">
-        <f t="shared" si="9"/>
+        <f t="shared" si="7"/>
         <v>167</v>
       </c>
       <c r="AH48">
-        <f t="shared" ref="AH48:AM48" si="10">AH46+AH47</f>
+        <f t="shared" ref="AH48:AM48" si="8">AH46+AH47</f>
         <v>357</v>
       </c>
       <c r="AI48">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>280</v>
       </c>
       <c r="AJ48">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>405</v>
       </c>
       <c r="AK48">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>928</v>
       </c>
       <c r="AL48">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>822</v>
       </c>
       <c r="AM48">
-        <f t="shared" si="10"/>
+        <f t="shared" si="8"/>
         <v>18685</v>
       </c>
     </row>
     <row r="49" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B49" s="8">
-        <f t="shared" ref="B49:AF49" si="11">B46/B48</f>
+        <f t="shared" ref="B49:AF49" si="9">B46/B48</f>
         <v>5.0880626223091974E-2</v>
       </c>
       <c r="C49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>6.6776586974443525E-2</v>
       </c>
       <c r="D49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.10128055878928988</v>
       </c>
       <c r="E49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.10861132660977502</v>
       </c>
       <c r="F49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.145985401459854</v>
       </c>
       <c r="G49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>9.878419452887538E-2</v>
       </c>
       <c r="H49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>2.5889967637540454E-2</v>
       </c>
       <c r="I49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>2.3456790123456792E-2</v>
       </c>
       <c r="J49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>4.3165467625899283E-2</v>
       </c>
       <c r="K49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>5.5079559363525092E-2</v>
       </c>
       <c r="L49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>6.397774687065369E-2</v>
       </c>
       <c r="M49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.17505809450038728</v>
       </c>
       <c r="N49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.15175953079178886</v>
       </c>
       <c r="O49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>8.0911233307148472E-2</v>
       </c>
       <c r="P49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.16243654822335024</v>
       </c>
       <c r="Q49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.13698630136986301</v>
       </c>
       <c r="R49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.17808219178082191</v>
       </c>
       <c r="S49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>4.7619047619047616E-2</v>
       </c>
       <c r="T49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="U49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.16190476190476191</v>
       </c>
       <c r="V49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.25531914893617019</v>
       </c>
       <c r="W49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.21428571428571427</v>
       </c>
       <c r="X49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.15094339622641509</v>
       </c>
       <c r="Y49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.21052631578947367</v>
       </c>
       <c r="Z49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.16113744075829384</v>
       </c>
       <c r="AA49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>9.0909090909090912E-2</v>
       </c>
       <c r="AB49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.1623931623931624</v>
       </c>
       <c r="AC49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>3.5294117647058823E-2</v>
       </c>
       <c r="AD49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.16883116883116883</v>
       </c>
       <c r="AE49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>0.29729729729729731</v>
       </c>
       <c r="AF49" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="9"/>
         <v>8.3832335329341312E-2</v>
       </c>
       <c r="AH49" s="8">
@@ -35734,155 +36272,155 @@
         <v>1533</v>
       </c>
       <c r="C78">
-        <f t="shared" ref="C78:AN78" si="12">SUM(C70:C77)</f>
+        <f t="shared" ref="C78:AN78" si="10">SUM(C70:C77)</f>
         <v>1213</v>
       </c>
       <c r="D78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>859</v>
       </c>
       <c r="E78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>1289</v>
       </c>
       <c r="F78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>959</v>
       </c>
       <c r="G78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>658</v>
       </c>
       <c r="H78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>618</v>
       </c>
       <c r="I78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>810</v>
       </c>
       <c r="J78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>695</v>
       </c>
       <c r="K78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>817</v>
       </c>
       <c r="L78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>719</v>
       </c>
       <c r="M78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>1291</v>
       </c>
       <c r="N78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>1364</v>
       </c>
       <c r="O78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>1273</v>
       </c>
       <c r="P78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>197</v>
       </c>
       <c r="Q78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>73</v>
       </c>
       <c r="R78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>146</v>
       </c>
       <c r="S78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>21</v>
       </c>
       <c r="T78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>48</v>
       </c>
       <c r="U78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>105</v>
       </c>
       <c r="V78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>47</v>
       </c>
       <c r="W78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>56</v>
       </c>
       <c r="X78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>53</v>
       </c>
       <c r="Y78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>38</v>
       </c>
       <c r="Z78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>211</v>
       </c>
       <c r="AA78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>55</v>
       </c>
       <c r="AB78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>2527</v>
       </c>
       <c r="AC78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>915</v>
       </c>
       <c r="AD78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>1070</v>
       </c>
       <c r="AE78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>117</v>
       </c>
       <c r="AF78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>85</v>
       </c>
       <c r="AG78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>154</v>
       </c>
       <c r="AH78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>222</v>
       </c>
       <c r="AI78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>167</v>
       </c>
       <c r="AJ78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>357</v>
       </c>
       <c r="AK78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>280</v>
       </c>
       <c r="AL78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>405</v>
       </c>
       <c r="AM78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>928</v>
       </c>
       <c r="AN78">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>822</v>
       </c>
       <c r="AO78">
@@ -35895,159 +36433,159 @@
         <v>568</v>
       </c>
       <c r="B79" s="1">
-        <f t="shared" ref="B79:B86" si="13">B70/B$78</f>
+        <f t="shared" ref="B79:B86" si="11">B70/B$78</f>
         <v>3.9138943248532287E-3</v>
       </c>
       <c r="C79" s="1">
-        <f t="shared" ref="C79:AN79" si="14">C70/C$78</f>
+        <f t="shared" ref="C79:AN79" si="12">C70/C$78</f>
         <v>8.2440230832646333E-4</v>
       </c>
       <c r="D79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>2.3282887077997671E-3</v>
       </c>
       <c r="E79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>4.1710114702815434E-3</v>
       </c>
       <c r="G79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="H79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="I79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>1.2345679012345679E-3</v>
       </c>
       <c r="J79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="K79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>2.4479804161566705E-3</v>
       </c>
       <c r="L79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="M79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>5.422153369481022E-3</v>
       </c>
       <c r="N79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>3.6656891495601175E-3</v>
       </c>
       <c r="O79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>1.5710919088766694E-3</v>
       </c>
       <c r="P79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Q79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>1.3698630136986301E-2</v>
       </c>
       <c r="R79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="S79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="U79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>2.8571428571428571E-2</v>
       </c>
       <c r="V79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="W79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="X79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Y79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="Z79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>4.7393364928909956E-3</v>
       </c>
       <c r="AA79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>1.8181818181818181E-2</v>
       </c>
       <c r="AB79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AC79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AD79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AE79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AF79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AG79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>1.2987012987012988E-2</v>
       </c>
       <c r="AH79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>9.0090090090090089E-3</v>
       </c>
       <c r="AI79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AJ79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AK79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AL79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="AM79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>2.1551724137931034E-3</v>
       </c>
       <c r="AN79" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
     </row>
@@ -36056,159 +36594,159 @@
         <v>129</v>
       </c>
       <c r="B80" s="1">
+        <f t="shared" si="11"/>
+        <v>6.5231572080887146E-4</v>
+      </c>
+      <c r="C80" s="1">
+        <f t="shared" ref="C80:AN86" si="13">C71/C$78</f>
+        <v>3.2976092333058533E-3</v>
+      </c>
+      <c r="D80" s="1">
         <f t="shared" si="13"/>
-        <v>6.5231572080887146E-4</v>
-      </c>
-      <c r="C80" s="1">
-        <f t="shared" ref="C80:AN86" si="15">C71/C$78</f>
-        <v>3.2976092333058533E-3</v>
-      </c>
-      <c r="D80" s="1">
-        <f t="shared" si="15"/>
         <v>3.4924330616996507E-3</v>
       </c>
       <c r="E80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.7579519006982156E-3</v>
       </c>
       <c r="F80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.2137643378519288E-3</v>
       </c>
       <c r="G80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.0790273556231003E-3</v>
       </c>
       <c r="H80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="I80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="J80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.4388489208633094E-3</v>
       </c>
       <c r="K80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="L80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.3908205841446453E-3</v>
       </c>
       <c r="M80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.2951200619674663E-3</v>
       </c>
       <c r="N80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.9325513196480938E-3</v>
       </c>
       <c r="O80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.8554595443833461E-3</v>
       </c>
       <c r="P80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.030456852791878E-2</v>
       </c>
       <c r="Q80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="R80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="S80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="U80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="V80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="W80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.7857142857142856E-2</v>
       </c>
       <c r="X80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Y80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Z80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AA80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.6363636363636362E-2</v>
       </c>
       <c r="AB80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AC80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AD80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.3457943925233649E-4</v>
       </c>
       <c r="AE80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.5470085470085479E-3</v>
       </c>
       <c r="AF80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.4935064935064939E-3</v>
       </c>
       <c r="AH80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.5045045045045043E-2</v>
       </c>
       <c r="AI80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AJ80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8011204481792717E-3</v>
       </c>
       <c r="AK80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.5714285714285713E-3</v>
       </c>
       <c r="AL80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.1551724137931034E-3</v>
       </c>
       <c r="AN80" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
@@ -36217,159 +36755,159 @@
         <v>130</v>
       </c>
       <c r="B81" s="1">
+        <f t="shared" si="11"/>
+        <v>0.94781474233529028</v>
+      </c>
+      <c r="C81" s="1">
+        <f t="shared" ref="C81:Q81" si="14">C72/C$78</f>
+        <v>0.93075020610057713</v>
+      </c>
+      <c r="D81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.89289871944121069</v>
+      </c>
+      <c r="E81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.88983708301008535</v>
+      </c>
+      <c r="F81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.84775808133472363</v>
+      </c>
+      <c r="G81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.89817629179331304</v>
+      </c>
+      <c r="H81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.96763754045307449</v>
+      </c>
+      <c r="I81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.97407407407407409</v>
+      </c>
+      <c r="J81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.94820143884892083</v>
+      </c>
+      <c r="K81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.94247246022031828</v>
+      </c>
+      <c r="L81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.93324061196105701</v>
+      </c>
+      <c r="M81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.82416731216111538</v>
+      </c>
+      <c r="N81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.84090909090909094</v>
+      </c>
+      <c r="O81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.91594658287509823</v>
+      </c>
+      <c r="P81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.8324873096446701</v>
+      </c>
+      <c r="Q81" s="1">
+        <f t="shared" si="14"/>
+        <v>0.86301369863013699</v>
+      </c>
+      <c r="R81" s="1">
         <f t="shared" si="13"/>
-        <v>0.94781474233529028</v>
-      </c>
-      <c r="C81" s="1">
-        <f t="shared" ref="C81:Q81" si="16">C72/C$78</f>
-        <v>0.93075020610057713</v>
-      </c>
-      <c r="D81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.89289871944121069</v>
-      </c>
-      <c r="E81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.88983708301008535</v>
-      </c>
-      <c r="F81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.84775808133472363</v>
-      </c>
-      <c r="G81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.89817629179331304</v>
-      </c>
-      <c r="H81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.96763754045307449</v>
-      </c>
-      <c r="I81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.97407407407407409</v>
-      </c>
-      <c r="J81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.94820143884892083</v>
-      </c>
-      <c r="K81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.94247246022031828</v>
-      </c>
-      <c r="L81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.93324061196105701</v>
-      </c>
-      <c r="M81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.82416731216111538</v>
-      </c>
-      <c r="N81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.84090909090909094</v>
-      </c>
-      <c r="O81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.91594658287509823</v>
-      </c>
-      <c r="P81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.8324873096446701</v>
-      </c>
-      <c r="Q81" s="1">
-        <f t="shared" si="16"/>
-        <v>0.86301369863013699</v>
-      </c>
-      <c r="R81" s="1">
-        <f t="shared" si="15"/>
         <v>0.81506849315068497</v>
       </c>
       <c r="S81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.90476190476190477</v>
       </c>
       <c r="T81" s="32">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.95833333333333337</v>
       </c>
       <c r="U81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.83809523809523812</v>
       </c>
       <c r="V81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.74468085106382975</v>
       </c>
       <c r="W81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.7857142857142857</v>
       </c>
       <c r="X81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.83018867924528306</v>
       </c>
       <c r="Y81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.78947368421052633</v>
       </c>
       <c r="Z81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.82938388625592419</v>
       </c>
       <c r="AA81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.90909090909090906</v>
       </c>
       <c r="AB81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.72734467748318166</v>
       </c>
       <c r="AC81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.65464480874316944</v>
       </c>
       <c r="AD81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.71588785046728975</v>
       </c>
       <c r="AE81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.83760683760683763</v>
       </c>
       <c r="AF81" s="32">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.96470588235294119</v>
       </c>
       <c r="AG81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.83116883116883122</v>
       </c>
       <c r="AH81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.68918918918918914</v>
       </c>
       <c r="AI81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.91616766467065869</v>
       </c>
       <c r="AJ81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.92156862745098034</v>
       </c>
       <c r="AK81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.93214285714285716</v>
       </c>
       <c r="AL81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.9555555555555556</v>
       </c>
       <c r="AM81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.93103448275862066</v>
       </c>
       <c r="AN81" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.93187347931873477</v>
       </c>
     </row>
@@ -36378,159 +36916,159 @@
         <v>131</v>
       </c>
       <c r="B82" s="1">
+        <f t="shared" si="11"/>
+        <v>2.6092628832354858E-3</v>
+      </c>
+      <c r="C82" s="1">
         <f t="shared" si="13"/>
-        <v>2.6092628832354858E-3</v>
-      </c>
-      <c r="C82" s="1">
-        <f t="shared" si="15"/>
         <v>1.236603462489695E-2</v>
       </c>
       <c r="D82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.1490104772991845E-3</v>
       </c>
       <c r="E82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.3964313421256789E-2</v>
       </c>
       <c r="F82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.2940563086548488E-2</v>
       </c>
       <c r="G82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.11854103343465E-3</v>
       </c>
       <c r="H82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.4724919093851136E-3</v>
       </c>
       <c r="I82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.4691358024691358E-3</v>
       </c>
       <c r="J82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.2949640287769784E-2</v>
       </c>
       <c r="K82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.4479804161566705E-3</v>
       </c>
       <c r="L82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.172461752433936E-3</v>
       </c>
       <c r="M82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.3237800154918668E-2</v>
       </c>
       <c r="N82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.6129032258064516E-2</v>
       </c>
       <c r="O82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.8554595443833461E-3</v>
       </c>
       <c r="P82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.5228426395939087E-2</v>
       </c>
       <c r="Q82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.7397260273972601E-2</v>
       </c>
       <c r="R82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.3698630136986301E-2</v>
       </c>
       <c r="S82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="U82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8571428571428571E-2</v>
       </c>
       <c r="V82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.2553191489361701E-2</v>
       </c>
       <c r="W82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.5714285714285712E-2</v>
       </c>
       <c r="X82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.5471698113207544E-2</v>
       </c>
       <c r="Y82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.10526315789473684</v>
       </c>
       <c r="Z82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.2654028436018961E-2</v>
       </c>
       <c r="AA82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AB82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.662049861495845E-2</v>
       </c>
       <c r="AC82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.8360655737704927E-3</v>
       </c>
       <c r="AD82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.6074766355140183E-3</v>
       </c>
       <c r="AE82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.564102564102564E-2</v>
       </c>
       <c r="AF82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.4935064935064939E-3</v>
       </c>
       <c r="AH82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.6036036036036036E-2</v>
       </c>
       <c r="AI82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AJ82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8011204481792717E-3</v>
       </c>
       <c r="AK82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AL82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.4691358024691358E-3</v>
       </c>
       <c r="AM82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.6206896551724137E-3</v>
       </c>
       <c r="AN82" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.8661800486618006E-3</v>
       </c>
     </row>
@@ -36539,159 +37077,159 @@
         <v>132</v>
       </c>
       <c r="B83" s="1">
+        <f t="shared" si="11"/>
+        <v>5.8708414872798431E-3</v>
+      </c>
+      <c r="C83" s="1">
         <f t="shared" si="13"/>
-        <v>5.8708414872798431E-3</v>
-      </c>
-      <c r="C83" s="1">
-        <f t="shared" si="15"/>
         <v>1.6488046166529267E-3</v>
       </c>
       <c r="D83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.3282887077997671E-3</v>
       </c>
       <c r="E83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.2063615205585725E-3</v>
       </c>
       <c r="F83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.2565172054223151E-3</v>
       </c>
       <c r="G83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.5197568389057751E-3</v>
       </c>
       <c r="H83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.6181229773462784E-3</v>
       </c>
       <c r="I83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.2345679012345679E-3</v>
       </c>
       <c r="J83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.4388489208633094E-3</v>
       </c>
       <c r="K83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.2239902080783353E-3</v>
       </c>
       <c r="L83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="M83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.422153369481022E-3</v>
       </c>
       <c r="N83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.9325513196480938E-3</v>
       </c>
       <c r="O83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.3566378633150041E-3</v>
       </c>
       <c r="P83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.015228426395939E-2</v>
       </c>
       <c r="Q83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="R83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="S83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="U83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.5238095238095247E-3</v>
       </c>
       <c r="V83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.1276595744680851E-2</v>
       </c>
       <c r="W83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="X83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Y83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Z83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AA83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AB83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.14364859517214087</v>
       </c>
       <c r="AC83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.12896174863387977</v>
       </c>
       <c r="AD83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.17570093457943925</v>
       </c>
       <c r="AE83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AF83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AG83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AH83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.5045045045045045E-3</v>
       </c>
       <c r="AI83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AJ83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8011204481792717E-3</v>
       </c>
       <c r="AK83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AL83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.387931034482759E-3</v>
       </c>
       <c r="AN83" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.4330900243309003E-3</v>
       </c>
     </row>
@@ -36700,159 +37238,159 @@
         <v>133</v>
       </c>
       <c r="B84" s="1">
+        <f t="shared" si="11"/>
+        <v>1.2393998695368558E-2</v>
+      </c>
+      <c r="C84" s="1">
         <f t="shared" si="13"/>
-        <v>1.2393998695368558E-2</v>
-      </c>
-      <c r="C84" s="1">
-        <f t="shared" si="15"/>
         <v>2.6380873866446827E-2</v>
       </c>
       <c r="D84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.8416763678696161E-2</v>
       </c>
       <c r="E84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.7323506594259115E-2</v>
       </c>
       <c r="F84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.3180396246089674E-2</v>
       </c>
       <c r="G84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.7355623100303952E-2</v>
       </c>
       <c r="H84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.4724919093851136E-3</v>
       </c>
       <c r="I84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.6419753086419745E-3</v>
       </c>
       <c r="J84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.0071942446043165E-2</v>
       </c>
       <c r="K84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.0807833537331701E-2</v>
       </c>
       <c r="L84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.6425591098748261E-2</v>
       </c>
       <c r="M84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.1967467079783116E-2</v>
       </c>
       <c r="N84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.8181818181818177E-2</v>
       </c>
       <c r="O84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.2780832678711706E-2</v>
       </c>
       <c r="P84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.5380710659898477E-2</v>
       </c>
       <c r="Q84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.3698630136986301E-2</v>
       </c>
       <c r="R84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.4246575342465752E-2</v>
       </c>
       <c r="S84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="T84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="U84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9047619047619049E-2</v>
       </c>
       <c r="V84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.10638297872340426</v>
       </c>
       <c r="W84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.10714285714285714</v>
       </c>
       <c r="X84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="Y84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.2631578947368418E-2</v>
       </c>
       <c r="Z84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.7393364928909949E-2</v>
       </c>
       <c r="AA84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.8181818181818181E-2</v>
       </c>
       <c r="AB84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.3240997229916899E-2</v>
       </c>
       <c r="AC84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.12568306010928962</v>
       </c>
       <c r="AD84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.1775700934579439E-2</v>
       </c>
       <c r="AE84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.8376068376068383E-2</v>
       </c>
       <c r="AF84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1764705882352941E-2</v>
       </c>
       <c r="AG84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.1428571428571425E-2</v>
       </c>
       <c r="AH84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.10810810810810811</v>
       </c>
       <c r="AI84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.9940119760479042E-2</v>
       </c>
       <c r="AJ84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.081232492997199E-2</v>
       </c>
       <c r="AK84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.4285714285714285E-2</v>
       </c>
       <c r="AL84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9753086419753086E-2</v>
       </c>
       <c r="AM84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.7241379310344827E-2</v>
       </c>
       <c r="AN84" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.0681265206812651E-2</v>
       </c>
     </row>
@@ -36861,159 +37399,159 @@
         <v>134</v>
       </c>
       <c r="B85" s="1">
+        <f t="shared" si="11"/>
+        <v>1.3698630136986301E-2</v>
+      </c>
+      <c r="C85" s="1">
         <f t="shared" si="13"/>
-        <v>1.3698630136986301E-2</v>
-      </c>
-      <c r="C85" s="1">
-        <f t="shared" si="15"/>
         <v>1.5663643858202802E-2</v>
       </c>
       <c r="D85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.9103608847497089E-2</v>
       </c>
       <c r="E85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.0170674941815361E-2</v>
       </c>
       <c r="F85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.3368091762252347E-2</v>
       </c>
       <c r="G85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8875379939209727E-2</v>
       </c>
       <c r="H85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.4724919093851136E-3</v>
       </c>
       <c r="I85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.4691358024691358E-3</v>
       </c>
       <c r="J85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.6330935251798559E-3</v>
       </c>
       <c r="K85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1015911872705019E-2</v>
       </c>
       <c r="L85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.2517385257301807E-2</v>
       </c>
       <c r="M85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.1123160340821067E-2</v>
       </c>
       <c r="N85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.398826979472141E-2</v>
       </c>
       <c r="O85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.5923016496465043E-2</v>
       </c>
       <c r="P85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.6142131979695438E-2</v>
       </c>
       <c r="Q85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.4794520547945202E-2</v>
       </c>
       <c r="R85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0.10273972602739725</v>
       </c>
       <c r="S85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.7619047619047616E-2</v>
       </c>
       <c r="T85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="U85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.7142857142857141E-2</v>
       </c>
       <c r="V85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>6.3829787234042548E-2</v>
       </c>
       <c r="W85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.5714285714285712E-2</v>
       </c>
       <c r="X85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.7735849056603772E-2</v>
       </c>
       <c r="Y85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.6315789473684209E-2</v>
       </c>
       <c r="Z85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.3175355450236969E-2</v>
       </c>
       <c r="AA85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.8181818181818181E-2</v>
       </c>
       <c r="AB85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.3027305104867431E-2</v>
       </c>
       <c r="AC85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.4644808743169397E-2</v>
       </c>
       <c r="AD85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.7943925233644861E-2</v>
       </c>
       <c r="AE85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.9829059829059832E-2</v>
       </c>
       <c r="AF85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1764705882352941E-2</v>
       </c>
       <c r="AG85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.1428571428571425E-2</v>
       </c>
       <c r="AH85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.2072072072072071E-2</v>
       </c>
       <c r="AI85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1976047904191617E-2</v>
       </c>
       <c r="AJ85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8011204481792717E-3</v>
       </c>
       <c r="AK85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>7.1428571428571426E-3</v>
       </c>
       <c r="AL85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AM85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9396551724137932E-2</v>
       </c>
       <c r="AN85" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>8.5158150851581509E-3</v>
       </c>
     </row>
@@ -37022,159 +37560,159 @@
         <v>135</v>
       </c>
       <c r="B86" s="1">
+        <f t="shared" si="11"/>
+        <v>1.3046314416177429E-2</v>
+      </c>
+      <c r="C86" s="1">
         <f t="shared" si="13"/>
-        <v>1.3046314416177429E-2</v>
-      </c>
-      <c r="C86" s="1">
-        <f t="shared" si="15"/>
         <v>9.0684253915910961E-3</v>
       </c>
       <c r="D86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.3282887077997673E-2</v>
       </c>
       <c r="E86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.4740108611326609E-2</v>
       </c>
       <c r="F86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.7111574556830033E-2</v>
       </c>
       <c r="G86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.8875379939209727E-2</v>
       </c>
       <c r="H86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1326860841423949E-2</v>
       </c>
       <c r="I86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>9.876543209876543E-3</v>
       </c>
       <c r="J86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.7266187050359712E-2</v>
       </c>
       <c r="K86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9583843329253364E-2</v>
       </c>
       <c r="L86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.2253129346314324E-2</v>
       </c>
       <c r="M86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9364833462432222E-2</v>
       </c>
       <c r="N86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.1260997067448679E-2</v>
       </c>
       <c r="O86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.5710919088766692E-2</v>
       </c>
       <c r="P86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.030456852791878E-2</v>
       </c>
       <c r="Q86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.7397260273972601E-2</v>
       </c>
       <c r="R86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.4246575342465752E-2</v>
       </c>
       <c r="S86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.7619047619047616E-2</v>
       </c>
       <c r="T86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="U86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.9047619047619049E-2</v>
       </c>
       <c r="V86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.1276595744680851E-2</v>
       </c>
       <c r="W86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.7857142857142856E-2</v>
       </c>
       <c r="X86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>5.6603773584905662E-2</v>
       </c>
       <c r="Y86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.6315789473684209E-2</v>
       </c>
       <c r="Z86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.2654028436018961E-2</v>
       </c>
       <c r="AA86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AB86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.6117926394934706E-2</v>
       </c>
       <c r="AC86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.6229508196721311E-2</v>
       </c>
       <c r="AD86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.2149532710280374E-2</v>
       </c>
       <c r="AE86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AF86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.1764705882352941E-2</v>
       </c>
       <c r="AG86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="AH86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.6036036036036036E-2</v>
       </c>
       <c r="AI86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.1916167664670656E-2</v>
       </c>
       <c r="AJ86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.6414565826330535E-2</v>
       </c>
       <c r="AK86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>4.2857142857142858E-2</v>
       </c>
       <c r="AL86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>2.2222222222222223E-2</v>
       </c>
       <c r="AM86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>1.4008620689655173E-2</v>
       </c>
       <c r="AN86" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="13"/>
         <v>3.1630170316301706E-2</v>
       </c>
     </row>
@@ -37254,15 +37792,15 @@
         <v>81</v>
       </c>
       <c r="G93" s="1">
-        <f t="shared" ref="G93:G137" si="17">F93/E93</f>
+        <f t="shared" ref="G93:G137" si="15">F93/E93</f>
         <v>6.6776586974443525E-2</v>
       </c>
       <c r="N93" t="str">
-        <f t="shared" ref="N93:N136" si="18">D93</f>
+        <f t="shared" ref="N93:N136" si="16">D93</f>
         <v>EXODUS</v>
       </c>
       <c r="O93" s="6">
-        <f t="shared" ref="O93:O136" si="19">G93</f>
+        <f t="shared" ref="O93:O136" si="17">G93</f>
         <v>6.6776586974443525E-2</v>
       </c>
     </row>
@@ -37283,15 +37821,15 @@
         <v>87</v>
       </c>
       <c r="G94" s="1">
+        <f t="shared" si="15"/>
+        <v>0.10128055878928988</v>
+      </c>
+      <c r="N94" t="str">
+        <f t="shared" si="16"/>
+        <v>LEVITICUS</v>
+      </c>
+      <c r="O94" s="6">
         <f t="shared" si="17"/>
-        <v>0.10128055878928988</v>
-      </c>
-      <c r="N94" t="str">
-        <f t="shared" si="18"/>
-        <v>LEVITICUS</v>
-      </c>
-      <c r="O94" s="6">
-        <f t="shared" si="19"/>
         <v>0.10128055878928988</v>
       </c>
     </row>
@@ -37312,15 +37850,15 @@
         <v>140</v>
       </c>
       <c r="G95" s="1">
+        <f t="shared" si="15"/>
+        <v>0.10861132660977502</v>
+      </c>
+      <c r="N95" t="str">
+        <f t="shared" si="16"/>
+        <v>NUMBERS</v>
+      </c>
+      <c r="O95" s="6">
         <f t="shared" si="17"/>
-        <v>0.10861132660977502</v>
-      </c>
-      <c r="N95" t="str">
-        <f t="shared" si="18"/>
-        <v>NUMBERS</v>
-      </c>
-      <c r="O95" s="6">
-        <f t="shared" si="19"/>
         <v>0.10861132660977502</v>
       </c>
     </row>
@@ -37341,7 +37879,7 @@
         <v>140</v>
       </c>
       <c r="G96" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.145985401459854</v>
       </c>
       <c r="I96" t="s">
@@ -37354,15 +37892,15 @@
         <v>140</v>
       </c>
       <c r="L96" s="1">
-        <f t="shared" ref="L96" si="20">K96/J96</f>
+        <f>K96/J96</f>
         <v>0.145985401459854</v>
       </c>
       <c r="N96" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>DEUTERONOMY</v>
       </c>
       <c r="O96" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.145985401459854</v>
       </c>
     </row>
@@ -37383,7 +37921,7 @@
         <v>65</v>
       </c>
       <c r="G97" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>9.878419452887538E-2</v>
       </c>
       <c r="I97" t="s">
@@ -37400,11 +37938,11 @@
         <v>0.16449086161879894</v>
       </c>
       <c r="N97" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>JOSHUA</v>
       </c>
       <c r="O97" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>9.878419452887538E-2</v>
       </c>
     </row>
@@ -37425,7 +37963,7 @@
         <v>17</v>
       </c>
       <c r="G98" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>2.7508090614886731E-2</v>
       </c>
       <c r="I98" t="s">
@@ -37438,15 +37976,15 @@
         <v>210</v>
       </c>
       <c r="L98" s="1">
-        <f t="shared" ref="L98:L117" si="21">K98/J98</f>
+        <f t="shared" ref="L98:L117" si="18">K98/J98</f>
         <v>0.15395894428152493</v>
       </c>
       <c r="N98" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>JUDGES</v>
       </c>
       <c r="O98" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>2.7508090614886731E-2</v>
       </c>
     </row>
@@ -37467,7 +38005,7 @@
         <v>19</v>
       </c>
       <c r="G99" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>2.3456790123456792E-2</v>
       </c>
       <c r="I99" t="s">
@@ -37480,15 +38018,15 @@
         <v>32</v>
       </c>
       <c r="L99" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.16243654822335024</v>
       </c>
       <c r="N99" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>1 SAMUEL</v>
       </c>
       <c r="O99" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>2.3456790123456792E-2</v>
       </c>
     </row>
@@ -37509,7 +38047,7 @@
         <v>30</v>
       </c>
       <c r="G100" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>4.3165467625899283E-2</v>
       </c>
       <c r="I100" t="s">
@@ -37522,15 +38060,15 @@
         <v>26</v>
       </c>
       <c r="L100" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.17808219178082191</v>
       </c>
       <c r="N100" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>2 SAMUEL</v>
       </c>
       <c r="O100" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>4.3165467625899283E-2</v>
       </c>
     </row>
@@ -37551,7 +38089,7 @@
         <v>45</v>
       </c>
       <c r="G101" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>5.5079559363525092E-2</v>
       </c>
       <c r="I101" t="s">
@@ -37564,15 +38102,15 @@
         <v>1</v>
       </c>
       <c r="L101" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>4.7619047619047616E-2</v>
       </c>
       <c r="N101" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>1 KINGS</v>
       </c>
       <c r="O101" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>5.5079559363525092E-2</v>
       </c>
     </row>
@@ -37593,7 +38131,7 @@
         <v>47</v>
       </c>
       <c r="G102" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>6.5368567454798326E-2</v>
       </c>
       <c r="I102" t="s">
@@ -37606,15 +38144,15 @@
         <v>17</v>
       </c>
       <c r="L102" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.16190476190476191</v>
       </c>
       <c r="N102" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>2 KINGS</v>
       </c>
       <c r="O102" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>6.5368567454798326E-2</v>
       </c>
     </row>
@@ -37628,7 +38166,7 @@
         <v>749</v>
       </c>
       <c r="G103" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>7.3647984267453295E-2</v>
       </c>
       <c r="I103" t="s">
@@ -37641,7 +38179,7 @@
         <v>12</v>
       </c>
       <c r="L103" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.25531914893617019</v>
       </c>
       <c r="O103" s="6"/>
@@ -37676,15 +38214,15 @@
         <v>12</v>
       </c>
       <c r="L104" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.21428571428571427</v>
       </c>
       <c r="N104" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>ISAIAH</v>
       </c>
       <c r="O104" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.16449086161879894</v>
       </c>
     </row>
@@ -37705,7 +38243,7 @@
         <v>210</v>
       </c>
       <c r="G105" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.15395894428152493</v>
       </c>
       <c r="I105" t="s">
@@ -37718,15 +38256,15 @@
         <v>8</v>
       </c>
       <c r="L105" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.15094339622641509</v>
       </c>
       <c r="N105" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>JEREMIAH</v>
       </c>
       <c r="O105" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.15395894428152493</v>
       </c>
     </row>
@@ -37747,7 +38285,7 @@
         <v>32</v>
       </c>
       <c r="G106" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.16243654822335024</v>
       </c>
       <c r="I106" t="s">
@@ -37760,15 +38298,15 @@
         <v>100</v>
       </c>
       <c r="L106" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.19047619047619047</v>
       </c>
       <c r="N106" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>HOSEA</v>
       </c>
       <c r="O106" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.16243654822335024</v>
       </c>
     </row>
@@ -37789,7 +38327,7 @@
         <v>26</v>
       </c>
       <c r="G107" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.17808219178082191</v>
       </c>
       <c r="I107" t="s">
@@ -37802,15 +38340,15 @@
         <v>104</v>
       </c>
       <c r="L107" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>8.1696779261586805E-2</v>
       </c>
       <c r="N107" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>AMOS</v>
       </c>
       <c r="O107" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.17808219178082191</v>
       </c>
     </row>
@@ -37831,7 +38369,7 @@
         <v>1</v>
       </c>
       <c r="G108" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>4.7619047619047616E-2</v>
       </c>
       <c r="I108" t="s">
@@ -37844,15 +38382,15 @@
         <v>10</v>
       </c>
       <c r="L108" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.13698630136986301</v>
       </c>
       <c r="N108" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>OBADIAH</v>
       </c>
       <c r="O108" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>4.7619047619047616E-2</v>
       </c>
     </row>
@@ -37873,7 +38411,7 @@
         <v>17</v>
       </c>
       <c r="G109" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.16190476190476191</v>
       </c>
       <c r="I109" t="s">
@@ -37886,15 +38424,15 @@
         <v>12</v>
       </c>
       <c r="L109" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.16666666666666666</v>
       </c>
       <c r="N109" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>MICAH</v>
       </c>
       <c r="O109" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.16190476190476191</v>
       </c>
     </row>
@@ -37915,7 +38453,7 @@
         <v>12</v>
       </c>
       <c r="G110" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.25531914893617019</v>
       </c>
       <c r="I110" t="s">
@@ -37928,15 +38466,15 @@
         <v>26</v>
       </c>
       <c r="L110" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.16883116883116883</v>
       </c>
       <c r="N110" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>NAHUM</v>
       </c>
       <c r="O110" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.25531914893617019</v>
       </c>
     </row>
@@ -37957,7 +38495,7 @@
         <v>12</v>
       </c>
       <c r="G111" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.21428571428571427</v>
       </c>
       <c r="I111" t="s">
@@ -37970,15 +38508,15 @@
         <v>8</v>
       </c>
       <c r="L111" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.21052631578947367</v>
       </c>
       <c r="N111" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>HABAKKUK</v>
       </c>
       <c r="O111" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.21428571428571427</v>
       </c>
     </row>
@@ -37999,7 +38537,7 @@
         <v>8</v>
       </c>
       <c r="G112" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.15094339622641509</v>
       </c>
       <c r="I112" t="s">
@@ -38012,15 +38550,15 @@
         <v>34</v>
       </c>
       <c r="L112" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.16113744075829384</v>
       </c>
       <c r="N112" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>ZEPHANIAH</v>
       </c>
       <c r="O112" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.15094339622641509</v>
       </c>
     </row>
@@ -38034,7 +38572,7 @@
         <v>444</v>
       </c>
       <c r="G113" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.16116152450090745</v>
       </c>
       <c r="I113" t="s">
@@ -38047,7 +38585,7 @@
         <v>19</v>
       </c>
       <c r="L113" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.1623931623931624</v>
       </c>
       <c r="O113" s="6"/>
@@ -38069,7 +38607,7 @@
         <v>100</v>
       </c>
       <c r="G114" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.19047619047619047</v>
       </c>
       <c r="I114" t="s">
@@ -38082,15 +38620,15 @@
         <v>66</v>
       </c>
       <c r="L114" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.29729729729729731</v>
       </c>
       <c r="N114" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>ISAIAH</v>
       </c>
       <c r="O114" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.19047619047619047</v>
       </c>
     </row>
@@ -38111,7 +38649,7 @@
         <v>104</v>
       </c>
       <c r="G115" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>8.1696779261586805E-2</v>
       </c>
       <c r="I115" t="s">
@@ -38124,15 +38662,15 @@
         <v>680</v>
       </c>
       <c r="L115" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.26909378709932724</v>
       </c>
       <c r="N115" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>EZEKIEL</v>
       </c>
       <c r="O115" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>8.1696779261586805E-2</v>
       </c>
     </row>
@@ -38153,7 +38691,7 @@
         <v>10</v>
       </c>
       <c r="G116" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.13698630136986301</v>
       </c>
       <c r="I116" t="s">
@@ -38166,15 +38704,15 @@
         <v>316</v>
       </c>
       <c r="L116" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.34535519125683062</v>
       </c>
       <c r="N116" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>JOEL</v>
       </c>
       <c r="O116" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.13698630136986301</v>
       </c>
     </row>
@@ -38195,7 +38733,7 @@
         <v>12</v>
       </c>
       <c r="G117" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.16666666666666666</v>
       </c>
       <c r="I117" t="s">
@@ -38208,15 +38746,15 @@
         <v>292</v>
       </c>
       <c r="L117" s="1">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>0.29258517034068138</v>
       </c>
       <c r="N117" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>JOB</v>
       </c>
       <c r="O117" s="6">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>0.16666666666666666</v>
       </c>
     </row>
@@ -38237,15 +38775,15 @@
         <v>26</v>
       </c>
       <c r="G118" s="1">
+        <f t="shared" si="15"/>
+        <v>0.16883116883116883</v>
+      </c>
+      <c r="N118" t="str">
+        <f t="shared" si="16"/>
+        <v>LAMENTATIONS</v>
+      </c>
+      <c r="O118" s="6">
         <f t="shared" si="17"/>
-        <v>0.16883116883116883</v>
-      </c>
-      <c r="N118" t="str">
-        <f t="shared" si="18"/>
-        <v>LAMENTATIONS</v>
-      </c>
-      <c r="O118" s="6">
-        <f t="shared" si="19"/>
         <v>0.16883116883116883</v>
       </c>
     </row>
@@ -38259,7 +38797,7 @@
         <v>252</v>
       </c>
       <c r="G119" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.12017167381974249</v>
       </c>
       <c r="O119" s="6"/>
@@ -38281,15 +38819,15 @@
         <v>2</v>
       </c>
       <c r="G120" s="1">
+        <f t="shared" si="15"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="N120" t="str">
+        <f t="shared" si="16"/>
+        <v>JONAH</v>
+      </c>
+      <c r="O120" s="6">
         <f t="shared" si="17"/>
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="N120" t="str">
-        <f t="shared" si="18"/>
-        <v>JONAH</v>
-      </c>
-      <c r="O120" s="6">
-        <f t="shared" si="19"/>
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
@@ -38310,15 +38848,15 @@
         <v>8</v>
       </c>
       <c r="G121" s="1">
+        <f t="shared" si="15"/>
+        <v>0.21052631578947367</v>
+      </c>
+      <c r="N121" t="str">
+        <f t="shared" si="16"/>
+        <v>HAGGAI</v>
+      </c>
+      <c r="O121" s="6">
         <f t="shared" si="17"/>
-        <v>0.21052631578947367</v>
-      </c>
-      <c r="N121" t="str">
-        <f t="shared" si="18"/>
-        <v>HAGGAI</v>
-      </c>
-      <c r="O121" s="6">
-        <f t="shared" si="19"/>
         <v>0.21052631578947367</v>
       </c>
     </row>
@@ -38339,15 +38877,15 @@
         <v>34</v>
       </c>
       <c r="G122" s="1">
+        <f t="shared" si="15"/>
+        <v>0.16113744075829384</v>
+      </c>
+      <c r="N122" t="str">
+        <f t="shared" si="16"/>
+        <v>ZECHARIAH</v>
+      </c>
+      <c r="O122" s="6">
         <f t="shared" si="17"/>
-        <v>0.16113744075829384</v>
-      </c>
-      <c r="N122" t="str">
-        <f t="shared" si="18"/>
-        <v>ZECHARIAH</v>
-      </c>
-      <c r="O122" s="6">
-        <f t="shared" si="19"/>
         <v>0.16113744075829384</v>
       </c>
     </row>
@@ -38368,15 +38906,15 @@
         <v>5</v>
       </c>
       <c r="G123" s="1">
+        <f t="shared" si="15"/>
+        <v>9.0909090909090912E-2</v>
+      </c>
+      <c r="N123" t="str">
+        <f t="shared" si="16"/>
+        <v>MALACHI</v>
+      </c>
+      <c r="O123" s="6">
         <f t="shared" si="17"/>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="N123" t="str">
-        <f t="shared" si="18"/>
-        <v>MALACHI</v>
-      </c>
-      <c r="O123" s="6">
-        <f t="shared" si="19"/>
         <v>9.0909090909090912E-2</v>
       </c>
     </row>
@@ -38397,15 +38935,15 @@
         <v>19</v>
       </c>
       <c r="G124" s="1">
+        <f t="shared" si="15"/>
+        <v>0.1623931623931624</v>
+      </c>
+      <c r="N124" t="str">
+        <f t="shared" si="16"/>
+        <v>SONG</v>
+      </c>
+      <c r="O124" s="6">
         <f t="shared" si="17"/>
-        <v>0.1623931623931624</v>
-      </c>
-      <c r="N124" t="str">
-        <f t="shared" si="18"/>
-        <v>SONG</v>
-      </c>
-      <c r="O124" s="6">
-        <f t="shared" si="19"/>
         <v>0.1623931623931624</v>
       </c>
     </row>
@@ -38426,15 +38964,15 @@
         <v>3</v>
       </c>
       <c r="G125" s="1">
+        <f t="shared" si="15"/>
+        <v>3.5294117647058823E-2</v>
+      </c>
+      <c r="N125" t="str">
+        <f t="shared" si="16"/>
+        <v>RUTH</v>
+      </c>
+      <c r="O125" s="6">
         <f t="shared" si="17"/>
-        <v>3.5294117647058823E-2</v>
-      </c>
-      <c r="N125" t="str">
-        <f t="shared" si="18"/>
-        <v>RUTH</v>
-      </c>
-      <c r="O125" s="6">
-        <f t="shared" si="19"/>
         <v>3.5294117647058823E-2</v>
       </c>
     </row>
@@ -38455,15 +38993,15 @@
         <v>66</v>
       </c>
       <c r="G126" s="1">
+        <f t="shared" si="15"/>
+        <v>0.29729729729729731</v>
+      </c>
+      <c r="N126" t="str">
+        <f t="shared" si="16"/>
+        <v>QOHELET</v>
+      </c>
+      <c r="O126" s="6">
         <f t="shared" si="17"/>
-        <v>0.29729729729729731</v>
-      </c>
-      <c r="N126" t="str">
-        <f t="shared" si="18"/>
-        <v>QOHELET</v>
-      </c>
-      <c r="O126" s="6">
-        <f t="shared" si="19"/>
         <v>0.29729729729729731</v>
       </c>
     </row>
@@ -38484,15 +39022,15 @@
         <v>14</v>
       </c>
       <c r="G127" s="1">
+        <f t="shared" si="15"/>
+        <v>8.3832335329341312E-2</v>
+      </c>
+      <c r="N127" t="str">
+        <f t="shared" si="16"/>
+        <v>ESTHER</v>
+      </c>
+      <c r="O127" s="6">
         <f t="shared" si="17"/>
-        <v>8.3832335329341312E-2</v>
-      </c>
-      <c r="N127" t="str">
-        <f t="shared" si="18"/>
-        <v>ESTHER</v>
-      </c>
-      <c r="O127" s="6">
-        <f t="shared" si="19"/>
         <v>8.3832335329341312E-2</v>
       </c>
     </row>
@@ -38513,15 +39051,15 @@
         <v>25</v>
       </c>
       <c r="G128" s="1">
+        <f t="shared" si="15"/>
+        <v>7.0028011204481794E-2</v>
+      </c>
+      <c r="N128" t="str">
+        <f t="shared" si="16"/>
+        <v>DANIEL</v>
+      </c>
+      <c r="O128" s="6">
         <f t="shared" si="17"/>
-        <v>7.0028011204481794E-2</v>
-      </c>
-      <c r="N128" t="str">
-        <f t="shared" si="18"/>
-        <v>DANIEL</v>
-      </c>
-      <c r="O128" s="6">
-        <f t="shared" si="19"/>
         <v>7.0028011204481794E-2</v>
       </c>
     </row>
@@ -38542,15 +39080,15 @@
         <v>16</v>
       </c>
       <c r="G129" s="1">
+        <f t="shared" si="15"/>
+        <v>5.7142857142857141E-2</v>
+      </c>
+      <c r="N129" t="str">
+        <f t="shared" si="16"/>
+        <v>EZRA</v>
+      </c>
+      <c r="O129" s="6">
         <f t="shared" si="17"/>
-        <v>5.7142857142857141E-2</v>
-      </c>
-      <c r="N129" t="str">
-        <f t="shared" si="18"/>
-        <v>EZRA</v>
-      </c>
-      <c r="O129" s="6">
-        <f t="shared" si="19"/>
         <v>5.7142857142857141E-2</v>
       </c>
     </row>
@@ -38571,15 +39109,15 @@
         <v>17</v>
       </c>
       <c r="G130" s="1">
+        <f t="shared" si="15"/>
+        <v>4.1975308641975309E-2</v>
+      </c>
+      <c r="N130" t="str">
+        <f t="shared" si="16"/>
+        <v>NEHEMIAH</v>
+      </c>
+      <c r="O130" s="6">
         <f t="shared" si="17"/>
-        <v>4.1975308641975309E-2</v>
-      </c>
-      <c r="N130" t="str">
-        <f t="shared" si="18"/>
-        <v>NEHEMIAH</v>
-      </c>
-      <c r="O130" s="6">
-        <f t="shared" si="19"/>
         <v>4.1975308641975309E-2</v>
       </c>
     </row>
@@ -38600,15 +39138,15 @@
         <v>59</v>
       </c>
       <c r="G131" s="1">
+        <f t="shared" si="15"/>
+        <v>6.3577586206896547E-2</v>
+      </c>
+      <c r="N131" t="str">
+        <f t="shared" si="16"/>
+        <v>1 CHRONICLES</v>
+      </c>
+      <c r="O131" s="6">
         <f t="shared" si="17"/>
-        <v>6.3577586206896547E-2</v>
-      </c>
-      <c r="N131" t="str">
-        <f t="shared" si="18"/>
-        <v>1 CHRONICLES</v>
-      </c>
-      <c r="O131" s="6">
-        <f t="shared" si="19"/>
         <v>6.3577586206896547E-2</v>
       </c>
     </row>
@@ -38629,15 +39167,15 @@
         <v>50</v>
       </c>
       <c r="G132" s="1">
+        <f t="shared" si="15"/>
+        <v>6.0827250608272508E-2</v>
+      </c>
+      <c r="N132" t="str">
+        <f t="shared" si="16"/>
+        <v>2 CHRONICLES</v>
+      </c>
+      <c r="O132" s="6">
         <f t="shared" si="17"/>
-        <v>6.0827250608272508E-2</v>
-      </c>
-      <c r="N132" t="str">
-        <f t="shared" si="18"/>
-        <v>2 CHRONICLES</v>
-      </c>
-      <c r="O132" s="6">
-        <f t="shared" si="19"/>
         <v>6.0827250608272508E-2</v>
       </c>
     </row>
@@ -38651,7 +39189,7 @@
         <v>318</v>
       </c>
       <c r="G133" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>8.514056224899598E-2</v>
       </c>
       <c r="O133" s="6"/>
@@ -38673,15 +39211,15 @@
         <v>680</v>
       </c>
       <c r="G134" s="1">
+        <f t="shared" si="15"/>
+        <v>0.26909378709932724</v>
+      </c>
+      <c r="N134" t="str">
+        <f t="shared" si="16"/>
+        <v>PSALMS</v>
+      </c>
+      <c r="O134" s="6">
         <f t="shared" si="17"/>
-        <v>0.26909378709932724</v>
-      </c>
-      <c r="N134" t="str">
-        <f t="shared" si="18"/>
-        <v>PSALMS</v>
-      </c>
-      <c r="O134" s="6">
-        <f t="shared" si="19"/>
         <v>0.26909378709932724</v>
       </c>
     </row>
@@ -38702,15 +39240,15 @@
         <v>316</v>
       </c>
       <c r="G135" s="1">
+        <f t="shared" si="15"/>
+        <v>0.34535519125683062</v>
+      </c>
+      <c r="N135" t="str">
+        <f t="shared" si="16"/>
+        <v>PROVERBS</v>
+      </c>
+      <c r="O135" s="6">
         <f t="shared" si="17"/>
-        <v>0.34535519125683062</v>
-      </c>
-      <c r="N135" t="str">
-        <f t="shared" si="18"/>
-        <v>PROVERBS</v>
-      </c>
-      <c r="O135" s="6">
-        <f t="shared" si="19"/>
         <v>0.34535519125683062</v>
       </c>
     </row>
@@ -38731,15 +39269,15 @@
         <v>292</v>
       </c>
       <c r="G136" s="1">
+        <f t="shared" si="15"/>
+        <v>0.29258517034068138</v>
+      </c>
+      <c r="N136" t="str">
+        <f t="shared" si="16"/>
+        <v>JOB</v>
+      </c>
+      <c r="O136" s="6">
         <f t="shared" si="17"/>
-        <v>0.29258517034068138</v>
-      </c>
-      <c r="N136" t="str">
-        <f t="shared" si="18"/>
-        <v>JOB</v>
-      </c>
-      <c r="O136" s="6">
-        <f t="shared" si="19"/>
         <v>0.29258517034068138</v>
       </c>
     </row>
@@ -38753,7 +39291,7 @@
         <v>1288</v>
       </c>
       <c r="G137" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.29009009009009007</v>
       </c>
     </row>
@@ -44008,7 +44546,7 @@
         <v>2097</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E5" si="0">C3/D3</f>
+        <f>C3/D3</f>
         <v>2.9566046733428709E-2</v>
       </c>
     </row>
@@ -44024,7 +44562,7 @@
         <v>3735</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="0"/>
+        <f>C4/D4</f>
         <v>2.7041499330655958E-2</v>
       </c>
     </row>
@@ -44040,7 +44578,7 @@
         <v>4440</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="0"/>
+        <f>C5/D5</f>
         <v>1.2837837837837839E-2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update psalm 37 translation
</commit_message>
<xml_diff>
--- a/musicscores/Openingnotes.xlsx
+++ b/musicscores/Openingnotes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1851" uniqueCount="751">
   <si>
     <t xml:space="preserve">e </t>
   </si>
@@ -2264,6 +2264,15 @@
   </si>
   <si>
     <t>Royalty</t>
+  </si>
+  <si>
+    <t>PNG size</t>
+  </si>
+  <si>
+    <t>for Kindle</t>
+  </si>
+  <si>
+    <t>For PB</t>
   </si>
 </sst>
 </file>
@@ -2431,7 +2440,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2472,6 +2481,7 @@
     <xf numFmtId="170" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
@@ -2805,11 +2815,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="222992384"/>
-        <c:axId val="187342144"/>
+        <c:axId val="222426624"/>
+        <c:axId val="249069568"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="222992384"/>
+        <c:axId val="222426624"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2818,7 +2828,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="187342144"/>
+        <c:crossAx val="249069568"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2826,7 +2836,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="187342144"/>
+        <c:axId val="249069568"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2837,7 +2847,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="222992384"/>
+        <c:crossAx val="222426624"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3181,11 +3191,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="223675904"/>
-        <c:axId val="223224384"/>
+        <c:axId val="222428672"/>
+        <c:axId val="249070720"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="223675904"/>
+        <c:axId val="222428672"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3194,7 +3204,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223224384"/>
+        <c:crossAx val="249070720"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3202,7 +3212,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="223224384"/>
+        <c:axId val="249070720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3213,7 +3223,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223675904"/>
+        <c:crossAx val="222428672"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3453,11 +3463,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="223676928"/>
-        <c:axId val="223226688"/>
+        <c:axId val="254400000"/>
+        <c:axId val="249073024"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="223676928"/>
+        <c:axId val="254400000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3466,7 +3476,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223226688"/>
+        <c:crossAx val="249073024"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3474,7 +3484,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="223226688"/>
+        <c:axId val="249073024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3485,7 +3495,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223676928"/>
+        <c:crossAx val="254400000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3882,11 +3892,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="223850496"/>
-        <c:axId val="223230144"/>
+        <c:axId val="254402048"/>
+        <c:axId val="249076480"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="223850496"/>
+        <c:axId val="254402048"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3895,7 +3905,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223230144"/>
+        <c:crossAx val="249076480"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3903,7 +3913,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="223230144"/>
+        <c:axId val="249076480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3914,7 +3924,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223850496"/>
+        <c:crossAx val="254402048"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4379,11 +4389,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="223674880"/>
-        <c:axId val="223231296"/>
+        <c:axId val="254401024"/>
+        <c:axId val="254967808"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="223674880"/>
+        <c:axId val="254401024"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4392,7 +4402,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223231296"/>
+        <c:crossAx val="254967808"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4400,7 +4410,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="223231296"/>
+        <c:axId val="254967808"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4411,7 +4421,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223674880"/>
+        <c:crossAx val="254401024"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4704,12 +4714,12 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:shape val="box"/>
-        <c:axId val="223853568"/>
-        <c:axId val="229444416"/>
+        <c:axId val="254905344"/>
+        <c:axId val="254971264"/>
         <c:axId val="0"/>
       </c:bar3DChart>
       <c:catAx>
-        <c:axId val="223853568"/>
+        <c:axId val="254905344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4718,7 +4728,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="229444416"/>
+        <c:crossAx val="254971264"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4726,7 +4736,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="229444416"/>
+        <c:axId val="254971264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4737,7 +4747,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="223853568"/>
+        <c:crossAx val="254905344"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5799,7 +5809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T67"/>
+  <dimension ref="A1:U67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -5816,7 +5826,7 @@
     <col min="20" max="20" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>73</v>
       </c>
@@ -5848,7 +5858,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>89</v>
       </c>
@@ -5859,7 +5869,7 @@
         <v>45778</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C3" s="14" t="s">
         <v>72</v>
       </c>
@@ -5875,46 +5885,55 @@
       <c r="G3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="14"/>
+      <c r="H3" s="14" t="s">
+        <v>140</v>
+      </c>
       <c r="I3" s="14" t="s">
+        <v>748</v>
+      </c>
+      <c r="J3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="K3" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="K3" s="14" t="s">
+      <c r="L3" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="L3" s="14"/>
-      <c r="Q3" t="s">
+      <c r="M3" s="14"/>
+      <c r="R3" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>140</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="9"/>
+      <c r="I4" s="8" t="s">
+        <v>749</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>750</v>
+      </c>
       <c r="K4" s="9"/>
-      <c r="M4" t="s">
+      <c r="L4" s="9"/>
+      <c r="N4" t="s">
         <v>81</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>88</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>137</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>83</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2245</v>
       </c>
@@ -5937,52 +5956,57 @@
       <c r="G5">
         <v>50</v>
       </c>
-      <c r="H5" s="8"/>
+      <c r="H5">
+        <v>2247</v>
+      </c>
       <c r="I5" s="10">
+        <v>34.200000000000003</v>
+      </c>
+      <c r="J5" s="10">
         <v>173.3</v>
       </c>
-      <c r="J5" s="17">
-        <f t="shared" ref="J5:J23" si="0">I5/A5</f>
+      <c r="K5" s="17">
+        <f>J5/A5</f>
         <v>7.7193763919821828E-2</v>
       </c>
-      <c r="K5" s="9">
+      <c r="L5" s="9">
         <f>A5/E5</f>
         <v>1.4644487932159165</v>
       </c>
-      <c r="L5" s="8">
+      <c r="M5" s="8">
         <f>E5/$E$23</f>
         <v>6.6088980858768756E-2</v>
       </c>
-      <c r="M5">
-        <f>S5-P5</f>
+      <c r="N5">
+        <f>T5-Q5</f>
         <v>39</v>
       </c>
-      <c r="N5" s="11">
-        <f t="shared" ref="N5:N11" si="1">ROUND(M5/E5,4)</f>
+      <c r="O5" s="11">
+        <f>ROUND(N5/E5,4)</f>
         <v>2.5399999999999999E-2</v>
       </c>
-      <c r="O5">
-        <f t="shared" ref="O5:O21" si="2">S5-P5</f>
+      <c r="P5">
+        <f t="shared" ref="P5:P21" si="0">T5-Q5</f>
         <v>39</v>
       </c>
-      <c r="P5" s="13">
+      <c r="Q5" s="13">
         <v>45710</v>
       </c>
-      <c r="Q5" s="13">
+      <c r="R5" s="13">
         <v>45719</v>
       </c>
-      <c r="R5" s="13">
+      <c r="S5" s="13">
         <v>45739</v>
       </c>
-      <c r="S5" s="13">
+      <c r="T5" s="13">
         <v>45749</v>
       </c>
-      <c r="T5" t="str">
+      <c r="U5" t="str">
         <f>C5</f>
         <v>Genesis</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1853</v>
       </c>
@@ -5999,58 +6023,63 @@
         <v>1213</v>
       </c>
       <c r="F6" s="10">
-        <f t="shared" ref="F6:F23" si="3">E6/D6</f>
+        <f t="shared" ref="F6:F23" si="1">E6/D6</f>
         <v>30.324999999999999</v>
       </c>
       <c r="G6">
         <v>40</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="10">
+      <c r="H6">
+        <v>1853</v>
+      </c>
+      <c r="I6" s="40">
+        <v>83.5</v>
+      </c>
+      <c r="J6" s="10">
         <v>143.5</v>
       </c>
-      <c r="J6" s="17">
+      <c r="K6" s="17">
+        <f>J6/A6</f>
+        <v>7.7441985968699403E-2</v>
+      </c>
+      <c r="L6" s="9">
+        <f>A6/E6</f>
+        <v>1.5276174773289366</v>
+      </c>
+      <c r="M6" s="8">
+        <f>E6/$E$23</f>
+        <v>5.2293498879117092E-2</v>
+      </c>
+      <c r="N6">
+        <f>T6-Q6</f>
+        <v>9</v>
+      </c>
+      <c r="O6" s="11">
+        <f>ROUND(N6/E6,4)</f>
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="P6">
         <f t="shared" si="0"/>
-        <v>7.7441985968699403E-2</v>
-      </c>
-      <c r="K6" s="9">
-        <f t="shared" ref="K6:K23" si="4">A6/E6</f>
-        <v>1.5276174773289366</v>
-      </c>
-      <c r="L6" s="8">
-        <f t="shared" ref="L6:L22" si="5">E6/$E$23</f>
-        <v>5.2293498879117092E-2</v>
-      </c>
-      <c r="M6">
-        <f>S6-P6</f>
         <v>9</v>
       </c>
-      <c r="N6" s="11">
-        <f t="shared" si="1"/>
-        <v>7.4000000000000003E-3</v>
-      </c>
-      <c r="O6">
-        <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
-      <c r="P6" s="13">
+      <c r="Q6" s="13">
         <v>45721</v>
       </c>
-      <c r="Q6" s="13">
+      <c r="R6" s="13">
         <v>45726</v>
       </c>
-      <c r="R6" s="13">
+      <c r="S6" s="13">
         <v>45722</v>
       </c>
-      <c r="S6" s="13">
+      <c r="T6" s="13">
         <v>45730</v>
       </c>
-      <c r="T6" t="str">
-        <f t="shared" ref="T6:T22" si="6">C6</f>
+      <c r="U6" t="str">
+        <f>C6</f>
         <v>Exodus</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1287</v>
       </c>
@@ -6067,58 +6096,63 @@
         <v>859</v>
       </c>
       <c r="F7" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>31.814814814814813</v>
       </c>
       <c r="G7">
         <v>27</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="10">
+      <c r="H7">
+        <v>1285</v>
+      </c>
+      <c r="I7" s="40">
+        <v>22</v>
+      </c>
+      <c r="J7" s="10">
         <v>100.7</v>
       </c>
-      <c r="J7" s="17">
+      <c r="K7" s="17">
+        <f>J7/A7</f>
+        <v>7.8243978243978246E-2</v>
+      </c>
+      <c r="L7" s="9">
+        <f>A7/E7</f>
+        <v>1.4982537834691503</v>
+      </c>
+      <c r="M7" s="8">
+        <f>E7/$E$23</f>
+        <v>3.7032246939127433E-2</v>
+      </c>
+      <c r="N7">
+        <f>T7-Q7</f>
+        <v>8</v>
+      </c>
+      <c r="O7" s="11">
+        <f>ROUND(N7/E7,4)</f>
+        <v>9.2999999999999992E-3</v>
+      </c>
+      <c r="P7">
         <f t="shared" si="0"/>
-        <v>7.8243978243978246E-2</v>
-      </c>
-      <c r="K7" s="9">
-        <f t="shared" si="4"/>
-        <v>1.4982537834691503</v>
-      </c>
-      <c r="L7" s="8">
-        <f t="shared" si="5"/>
-        <v>3.7032246939127433E-2</v>
-      </c>
-      <c r="M7">
-        <f>S7-P7</f>
         <v>8</v>
       </c>
-      <c r="N7" s="11">
-        <f t="shared" si="1"/>
-        <v>9.2999999999999992E-3</v>
-      </c>
-      <c r="O7">
-        <f t="shared" si="2"/>
-        <v>8</v>
-      </c>
-      <c r="P7" s="13">
+      <c r="Q7" s="13">
         <v>45769</v>
       </c>
-      <c r="Q7" s="13">
+      <c r="R7" s="13">
         <v>45776</v>
       </c>
-      <c r="R7" s="13">
+      <c r="S7" s="13">
         <v>45768</v>
       </c>
-      <c r="S7" s="13">
+      <c r="T7" s="13">
         <v>45777</v>
       </c>
-      <c r="T7" t="str">
-        <f t="shared" si="6"/>
+      <c r="U7" t="str">
+        <f>C7</f>
         <v>Leviticus</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1855</v>
       </c>
@@ -6135,58 +6169,63 @@
         <v>1288</v>
       </c>
       <c r="F8" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>35.777777777777779</v>
       </c>
       <c r="G8">
         <v>36</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="10">
+      <c r="H8">
+        <v>1853</v>
+      </c>
+      <c r="I8" s="40">
+        <v>29.1</v>
+      </c>
+      <c r="J8" s="10">
         <v>143.30000000000001</v>
       </c>
-      <c r="J8" s="17">
+      <c r="K8" s="17">
+        <f>J8/A8</f>
+        <v>7.7250673854447449E-2</v>
+      </c>
+      <c r="L8" s="9">
+        <f>A8/E8</f>
+        <v>1.4402173913043479</v>
+      </c>
+      <c r="M8" s="8">
+        <f>E8/$E$23</f>
+        <v>5.552681496809795E-2</v>
+      </c>
+      <c r="N8">
+        <f t="shared" ref="N8:N22" si="2">T8-Q8</f>
+        <v>6</v>
+      </c>
+      <c r="O8" s="11">
+        <f>ROUND(N8/E8,4)</f>
+        <v>4.7000000000000002E-3</v>
+      </c>
+      <c r="P8">
         <f t="shared" si="0"/>
-        <v>7.7250673854447449E-2</v>
-      </c>
-      <c r="K8" s="9">
-        <f t="shared" si="4"/>
-        <v>1.4402173913043479</v>
-      </c>
-      <c r="L8" s="8">
-        <f t="shared" si="5"/>
-        <v>5.552681496809795E-2</v>
-      </c>
-      <c r="M8">
-        <f t="shared" ref="M8:M22" si="7">S8-P8</f>
         <v>6</v>
       </c>
-      <c r="N8" s="11">
-        <f t="shared" si="1"/>
-        <v>4.7000000000000002E-3</v>
-      </c>
-      <c r="O8">
-        <f t="shared" si="2"/>
-        <v>6</v>
-      </c>
-      <c r="P8" s="13">
+      <c r="Q8" s="13">
         <v>45778</v>
       </c>
-      <c r="Q8" s="13">
+      <c r="R8" s="13">
         <v>45783</v>
       </c>
-      <c r="R8" s="13">
+      <c r="S8" s="13">
         <v>45778</v>
       </c>
-      <c r="S8" s="13">
+      <c r="T8" s="13">
         <v>45784</v>
       </c>
-      <c r="T8" t="str">
-        <f t="shared" si="6"/>
+      <c r="U8" t="str">
+        <f>C8</f>
         <v>Numbers</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1553</v>
       </c>
@@ -6203,58 +6242,63 @@
         <v>959</v>
       </c>
       <c r="F9" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>28.205882352941178</v>
       </c>
       <c r="G9">
         <v>34</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="10">
+      <c r="H9">
+        <v>1565</v>
+      </c>
+      <c r="I9" s="40">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="J9" s="10">
         <v>123.1</v>
       </c>
-      <c r="J9" s="17">
-        <f t="shared" si="0"/>
+      <c r="K9" s="17">
+        <f>J9/A9</f>
         <v>7.9265936896329686E-2</v>
       </c>
-      <c r="K9" s="9">
-        <f t="shared" si="4"/>
+      <c r="L9" s="9">
+        <f>A9/E9</f>
         <v>1.6193952033368091</v>
       </c>
-      <c r="L9" s="8">
-        <f t="shared" si="5"/>
+      <c r="M9" s="8">
+        <f>E9/$E$23</f>
         <v>4.1343335057768583E-2</v>
       </c>
-      <c r="M9">
-        <f t="shared" si="7"/>
-        <v>28</v>
-      </c>
-      <c r="N9" s="11">
-        <f t="shared" si="1"/>
-        <v>2.92E-2</v>
-      </c>
-      <c r="O9">
+      <c r="N9">
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
-      <c r="P9" s="13">
+      <c r="O9" s="11">
+        <f>ROUND(N9/E9,4)</f>
+        <v>2.92E-2</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="Q9" s="13">
         <v>45659</v>
       </c>
-      <c r="Q9" s="13">
+      <c r="R9" s="13">
         <v>45686</v>
       </c>
-      <c r="R9" s="13">
+      <c r="S9" s="13">
         <v>45657</v>
       </c>
-      <c r="S9" s="13">
+      <c r="T9" s="13">
         <v>45687</v>
       </c>
-      <c r="T9" t="str">
-        <f t="shared" si="6"/>
+      <c r="U9" t="str">
+        <f>C9</f>
         <v>Deuteronomy</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2148</v>
       </c>
@@ -6271,52 +6315,57 @@
         <v>1276</v>
       </c>
       <c r="F10" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>28.355555555555554</v>
       </c>
       <c r="G10">
         <v>45</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="10">
+      <c r="H10">
+        <v>2146</v>
+      </c>
+      <c r="I10" s="40">
+        <v>33.6</v>
+      </c>
+      <c r="J10" s="10">
         <v>158</v>
       </c>
-      <c r="J10" s="17">
-        <f t="shared" si="0"/>
+      <c r="K10" s="17">
+        <f>J10/A10</f>
         <v>7.3556797020484177E-2</v>
       </c>
-      <c r="K10" s="9">
-        <f t="shared" si="4"/>
+      <c r="L10" s="9">
+        <f>A10/E10</f>
         <v>1.6833855799373041</v>
       </c>
-      <c r="L10" s="8">
-        <f t="shared" si="5"/>
+      <c r="M10" s="8">
+        <f>E10/$E$23</f>
         <v>5.5009484393861011E-2</v>
       </c>
-      <c r="M10">
-        <f t="shared" si="7"/>
-        <v>16</v>
-      </c>
-      <c r="N10" s="11">
-        <f t="shared" si="1"/>
-        <v>1.2500000000000001E-2</v>
-      </c>
-      <c r="O10">
+      <c r="N10">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="P10" s="13">
+      <c r="O10" s="11">
+        <f>ROUND(N10/E10,4)</f>
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="Q10" s="13">
         <v>45820</v>
       </c>
-      <c r="S10" s="13">
+      <c r="T10" s="13">
         <v>45836</v>
       </c>
-      <c r="T10" t="str">
-        <f t="shared" si="6"/>
+      <c r="U10" t="str">
+        <f>C10</f>
         <v>Joshua, Judges</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2560</v>
       </c>
@@ -6333,52 +6382,57 @@
         <v>1505</v>
       </c>
       <c r="F11" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>27.363636363636363</v>
       </c>
       <c r="G11">
         <v>55</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="10">
+      <c r="H11">
+        <v>2558</v>
+      </c>
+      <c r="I11" s="40">
+        <v>39</v>
+      </c>
+      <c r="J11" s="10">
         <v>186.7</v>
       </c>
-      <c r="J11" s="17">
-        <f t="shared" si="0"/>
+      <c r="K11" s="17">
+        <f>J11/A11</f>
         <v>7.2929687499999993E-2</v>
       </c>
-      <c r="K11" s="9">
-        <f t="shared" si="4"/>
+      <c r="L11" s="9">
+        <f>A11/E11</f>
         <v>1.7009966777408638</v>
       </c>
-      <c r="L11" s="8">
-        <f t="shared" si="5"/>
+      <c r="M11" s="8">
+        <f>E11/$E$23</f>
         <v>6.4881876185549234E-2</v>
       </c>
-      <c r="M11">
-        <f t="shared" si="7"/>
-        <v>18</v>
-      </c>
-      <c r="N11" s="11">
-        <f t="shared" si="1"/>
-        <v>1.2E-2</v>
-      </c>
-      <c r="O11">
+      <c r="N11">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="P11" s="13">
+      <c r="O11" s="11">
+        <f>ROUND(N11/E11,4)</f>
+        <v>1.2E-2</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="Q11" s="13">
         <v>45836</v>
       </c>
-      <c r="S11" s="13">
+      <c r="T11" s="13">
         <v>45854</v>
       </c>
-      <c r="T11" t="str">
-        <f t="shared" si="6"/>
+      <c r="U11" t="str">
+        <f>C11</f>
         <v>Samuel</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2705</v>
       </c>
@@ -6395,58 +6449,63 @@
         <v>1536</v>
       </c>
       <c r="F12" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>32.680851063829785</v>
       </c>
       <c r="G12">
         <v>47</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="10">
+      <c r="H12">
+        <v>2703</v>
+      </c>
+      <c r="I12" s="40">
+        <v>41</v>
+      </c>
+      <c r="J12" s="10">
         <v>198.1</v>
       </c>
-      <c r="J12" s="17">
-        <f t="shared" si="0"/>
+      <c r="K12" s="17">
+        <f>J12/A12</f>
         <v>7.3234750462107201E-2</v>
       </c>
-      <c r="K12" s="9">
-        <f t="shared" si="4"/>
+      <c r="L12" s="9">
+        <f>A12/E12</f>
         <v>1.7610677083333333</v>
       </c>
-      <c r="L12" s="8">
-        <f t="shared" si="5"/>
+      <c r="M12" s="8">
+        <f>E12/$E$23</f>
         <v>6.6218313502327986E-2</v>
       </c>
-      <c r="M12">
-        <f t="shared" si="7"/>
-        <v>16</v>
-      </c>
-      <c r="N12" s="11">
-        <f t="shared" ref="N12:N20" si="8">ROUND(M12/E12,4)</f>
-        <v>1.04E-2</v>
-      </c>
-      <c r="O12">
+      <c r="N12">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="P12" s="13">
+      <c r="O12" s="11">
+        <f>ROUND(N12/E12,4)</f>
+        <v>1.04E-2</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="Q12" s="13">
         <v>45796</v>
       </c>
-      <c r="Q12" s="13">
+      <c r="R12" s="13">
         <v>45811</v>
       </c>
-      <c r="R12" s="13">
+      <c r="S12" s="13">
         <v>45796</v>
       </c>
-      <c r="S12" s="13">
+      <c r="T12" s="13">
         <v>45812</v>
       </c>
-      <c r="T12" t="str">
-        <f t="shared" si="6"/>
+      <c r="U12" t="str">
+        <f>C12</f>
         <v>Kings</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1903</v>
       </c>
@@ -6463,58 +6522,63 @@
         <v>1291</v>
       </c>
       <c r="F13" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>19.560606060606062</v>
       </c>
       <c r="G13">
         <v>66</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="10">
+      <c r="H13">
+        <v>1917</v>
+      </c>
+      <c r="I13" s="40">
+        <v>110.9</v>
+      </c>
+      <c r="J13" s="10">
         <v>135.19999999999999</v>
       </c>
-      <c r="J13" s="17">
-        <f t="shared" si="0"/>
+      <c r="K13" s="17">
+        <f>J13/A13</f>
         <v>7.104571728849185E-2</v>
       </c>
-      <c r="K13" s="9">
-        <f t="shared" si="4"/>
+      <c r="L13" s="9">
+        <f>A13/E13</f>
         <v>1.4740511231603408</v>
       </c>
-      <c r="L13" s="8">
-        <f t="shared" si="5"/>
+      <c r="M13" s="8">
+        <f>E13/$E$23</f>
         <v>5.5656147611657179E-2</v>
       </c>
-      <c r="M13">
-        <f t="shared" si="7"/>
-        <v>23</v>
-      </c>
-      <c r="N13" s="11">
-        <f t="shared" si="8"/>
-        <v>1.78E-2</v>
-      </c>
-      <c r="O13">
+      <c r="N13">
         <f t="shared" si="2"/>
         <v>23</v>
       </c>
-      <c r="P13" s="13">
+      <c r="O13" s="11">
+        <f>ROUND(N13/E13,4)</f>
+        <v>1.78E-2</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="Q13" s="13">
         <v>45699</v>
       </c>
-      <c r="Q13" s="13">
+      <c r="R13" s="13">
         <v>45726</v>
       </c>
-      <c r="R13" s="13">
+      <c r="S13" s="13">
         <v>45698</v>
       </c>
-      <c r="S13" s="13">
+      <c r="T13" s="13">
         <v>45722</v>
       </c>
-      <c r="T13" t="str">
-        <f t="shared" si="6"/>
+      <c r="U13" t="str">
+        <f>C13</f>
         <v>Isaiah</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2318</v>
       </c>
@@ -6531,58 +6595,63 @@
         <v>1364</v>
       </c>
       <c r="F14" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>26.23076923076923</v>
       </c>
       <c r="G14">
         <v>52</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="10">
+      <c r="H14">
+        <v>2316</v>
+      </c>
+      <c r="I14" s="40">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="J14" s="10">
         <v>168.9</v>
       </c>
-      <c r="J14" s="17">
-        <f t="shared" si="0"/>
+      <c r="K14" s="17">
+        <f>J14/A14</f>
         <v>7.2864538395168252E-2</v>
       </c>
-      <c r="K14" s="9">
-        <f t="shared" si="4"/>
+      <c r="L14" s="9">
+        <f>A14/E14</f>
         <v>1.6994134897360704</v>
       </c>
-      <c r="L14" s="8">
-        <f t="shared" si="5"/>
+      <c r="M14" s="8">
+        <f>E14/$E$23</f>
         <v>5.8803241938265222E-2</v>
       </c>
-      <c r="M14">
-        <f t="shared" si="7"/>
-        <v>13</v>
-      </c>
-      <c r="N14" s="11">
-        <f t="shared" si="8"/>
-        <v>9.4999999999999998E-3</v>
-      </c>
-      <c r="O14">
+      <c r="N14">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="P14" s="13">
+      <c r="O14" s="11">
+        <f>ROUND(N14/E14,4)</f>
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="Q14" s="13">
         <v>45751</v>
       </c>
-      <c r="Q14" s="13">
+      <c r="R14" s="13">
         <v>45764</v>
       </c>
-      <c r="R14" s="13">
+      <c r="S14" s="13">
         <v>45751</v>
       </c>
-      <c r="S14" s="13">
+      <c r="T14" s="13">
         <v>45764</v>
       </c>
-      <c r="T14" t="str">
-        <f t="shared" si="6"/>
+      <c r="U14" t="str">
+        <f>C14</f>
         <v>Jeremiah</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2066</v>
       </c>
@@ -6599,58 +6668,63 @@
         <v>1273</v>
       </c>
       <c r="F15" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>26.520833333333332</v>
       </c>
       <c r="G15">
         <v>48</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="10">
+      <c r="H15">
+        <v>2064</v>
+      </c>
+      <c r="I15" s="40">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="J15" s="10">
         <v>149.80000000000001</v>
       </c>
-      <c r="J15" s="17">
-        <f t="shared" si="0"/>
+      <c r="K15" s="17">
+        <f>J15/A15</f>
         <v>7.2507260406582771E-2</v>
       </c>
-      <c r="K15" s="9">
-        <f t="shared" si="4"/>
+      <c r="L15" s="9">
+        <f>A15/E15</f>
         <v>1.6229379418695993</v>
       </c>
-      <c r="L15" s="8">
-        <f t="shared" si="5"/>
+      <c r="M15" s="8">
+        <f>E15/$E$23</f>
         <v>5.4880151750301774E-2</v>
       </c>
-      <c r="M15">
-        <f t="shared" si="7"/>
-        <v>12</v>
-      </c>
-      <c r="N15" s="11">
-        <f t="shared" si="8"/>
-        <v>9.4000000000000004E-3</v>
-      </c>
-      <c r="O15">
+      <c r="N15">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="P15" s="13">
+      <c r="O15" s="11">
+        <f>ROUND(N15/E15,4)</f>
+        <v>9.4000000000000004E-3</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="Q15" s="13">
         <v>45784</v>
       </c>
-      <c r="Q15" s="13">
+      <c r="R15" s="13">
         <v>45796</v>
       </c>
-      <c r="R15" s="13">
+      <c r="S15" s="13">
         <v>45784</v>
       </c>
-      <c r="S15" s="13">
+      <c r="T15" s="13">
         <v>45796</v>
       </c>
-      <c r="T15" t="str">
-        <f t="shared" si="6"/>
+      <c r="U15" t="str">
+        <f>C15</f>
         <v>Ezekiel</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1583</v>
       </c>
@@ -6667,58 +6741,63 @@
         <v>1050</v>
       </c>
       <c r="F16" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>15.671641791044776</v>
       </c>
       <c r="G16">
         <v>67</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="10">
+      <c r="H16">
+        <v>1583</v>
+      </c>
+      <c r="I16" s="40">
+        <v>77.599999999999994</v>
+      </c>
+      <c r="J16" s="10">
         <v>122.7</v>
       </c>
-      <c r="J16" s="17">
-        <f t="shared" si="0"/>
+      <c r="K16" s="17">
+        <f>J16/A16</f>
         <v>7.751105495893873E-2</v>
       </c>
-      <c r="K16" s="9">
-        <f t="shared" si="4"/>
+      <c r="L16" s="9">
+        <f>A16/E16</f>
         <v>1.5076190476190476</v>
       </c>
-      <c r="L16" s="8">
-        <f t="shared" si="5"/>
+      <c r="M16" s="8">
+        <f>E16/$E$23</f>
         <v>4.5266425245732024E-2</v>
       </c>
-      <c r="M16">
-        <f t="shared" si="7"/>
-        <v>7</v>
-      </c>
-      <c r="N16" s="11">
-        <f t="shared" si="8"/>
-        <v>6.7000000000000002E-3</v>
-      </c>
-      <c r="O16">
+      <c r="N16">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="P16" s="13">
+      <c r="O16" s="11">
+        <f>ROUND(N16/E16,4)</f>
+        <v>6.7000000000000002E-3</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="Q16" s="13">
         <v>45731</v>
       </c>
-      <c r="Q16" s="13">
+      <c r="R16" s="13">
         <v>45738</v>
       </c>
-      <c r="R16" s="13">
+      <c r="S16" s="13">
         <v>45731</v>
       </c>
-      <c r="S16" s="13">
+      <c r="T16" s="13">
         <v>45738</v>
       </c>
-      <c r="T16" t="str">
-        <f t="shared" si="6"/>
+      <c r="U16" t="str">
+        <f>C16</f>
         <v>The Twelve</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2604</v>
       </c>
@@ -6735,58 +6814,63 @@
         <v>2527</v>
       </c>
       <c r="F17" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>16.846666666666668</v>
       </c>
       <c r="G17">
         <v>150</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="10">
+      <c r="H17">
+        <v>2602</v>
+      </c>
+      <c r="I17" s="40">
+        <v>36.5</v>
+      </c>
+      <c r="J17" s="10">
         <v>227</v>
       </c>
-      <c r="J17" s="17">
-        <f t="shared" si="0"/>
+      <c r="K17" s="17">
+        <f>J17/A17</f>
         <v>8.7173579109062982E-2</v>
       </c>
-      <c r="K17" s="9">
-        <f t="shared" si="4"/>
+      <c r="L17" s="9">
+        <f>A17/E17</f>
         <v>1.0304709141274238</v>
       </c>
-      <c r="L17" s="8">
-        <f t="shared" si="5"/>
+      <c r="M17" s="8">
+        <f>E17/$E$23</f>
         <v>0.10894119675806173</v>
       </c>
-      <c r="M17">
-        <f t="shared" si="7"/>
-        <v>15</v>
-      </c>
-      <c r="N17" s="11">
-        <f t="shared" si="8"/>
-        <v>5.8999999999999999E-3</v>
-      </c>
-      <c r="O17">
+      <c r="N17">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="P17" s="13">
+      <c r="O17" s="11">
+        <f>ROUND(N17/E17,4)</f>
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="Q17" s="13">
         <v>45682</v>
       </c>
-      <c r="Q17" s="13">
+      <c r="R17" s="13">
         <v>45695</v>
       </c>
-      <c r="R17" s="13">
+      <c r="S17" s="13">
         <v>45668</v>
       </c>
-      <c r="S17" s="13">
+      <c r="T17" s="13">
         <v>45697</v>
       </c>
-      <c r="T17" t="str">
-        <f t="shared" si="6"/>
+      <c r="U17" t="str">
+        <f>C17</f>
         <v>Psalms</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>920</v>
       </c>
@@ -6803,58 +6887,63 @@
         <v>915</v>
       </c>
       <c r="F18" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>29.516129032258064</v>
       </c>
       <c r="G18">
         <v>31</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="10">
+      <c r="H18">
+        <v>918</v>
+      </c>
+      <c r="I18" s="40">
+        <v>15.9</v>
+      </c>
+      <c r="J18" s="10">
         <v>58</v>
       </c>
-      <c r="J18" s="17">
-        <f t="shared" si="0"/>
+      <c r="K18" s="17">
+        <f>J18/A18</f>
         <v>6.3043478260869562E-2</v>
       </c>
-      <c r="K18" s="9">
-        <f t="shared" si="4"/>
+      <c r="L18" s="9">
+        <f>A18/E18</f>
         <v>1.0054644808743169</v>
       </c>
-      <c r="L18" s="8">
-        <f t="shared" si="5"/>
+      <c r="M18" s="8">
+        <f>E18/$E$23</f>
         <v>3.9446456285566478E-2</v>
       </c>
-      <c r="M18">
-        <f t="shared" si="7"/>
-        <v>5</v>
-      </c>
-      <c r="N18" s="11">
-        <f t="shared" si="8"/>
-        <v>5.4999999999999997E-3</v>
-      </c>
-      <c r="O18">
+      <c r="N18">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="P18" s="13">
+      <c r="O18" s="11">
+        <f>ROUND(N18/E18,4)</f>
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="Q18" s="13">
         <v>45764</v>
       </c>
-      <c r="Q18" s="13">
+      <c r="R18" s="13">
         <v>45767</v>
       </c>
-      <c r="R18" s="13">
+      <c r="S18" s="13">
         <v>45766</v>
       </c>
-      <c r="S18" s="13">
+      <c r="T18" s="13">
         <v>45769</v>
       </c>
-      <c r="T18" t="str">
-        <f t="shared" si="6"/>
+      <c r="U18" t="str">
+        <f>C18</f>
         <v>Proverbs</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1279</v>
       </c>
@@ -6871,58 +6960,63 @@
         <v>1070</v>
       </c>
       <c r="F19" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>25.476190476190474</v>
       </c>
       <c r="G19">
         <v>42</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="10">
+      <c r="H19">
+        <v>1203</v>
+      </c>
+      <c r="I19" s="40">
+        <v>37.6</v>
+      </c>
+      <c r="J19" s="10">
         <v>105.4</v>
       </c>
-      <c r="J19" s="17">
-        <f t="shared" si="0"/>
+      <c r="K19" s="17">
+        <f>J19/A19</f>
         <v>8.2408131352619235E-2</v>
       </c>
-      <c r="K19" s="9">
-        <f t="shared" si="4"/>
+      <c r="L19" s="9">
+        <f>A19/E19</f>
         <v>1.1953271028037382</v>
       </c>
-      <c r="L19" s="8">
-        <f t="shared" si="5"/>
+      <c r="M19" s="8">
+        <f>E19/$E$23</f>
         <v>4.6128642869460251E-2</v>
       </c>
-      <c r="M19">
-        <f t="shared" si="7"/>
-        <v>33</v>
-      </c>
-      <c r="N19" s="11">
-        <f t="shared" si="8"/>
-        <v>3.0800000000000001E-2</v>
-      </c>
-      <c r="O19">
+      <c r="N19">
         <f t="shared" si="2"/>
         <v>33</v>
       </c>
-      <c r="P19" s="13">
+      <c r="O19" s="11">
+        <f>ROUND(N19/E19,4)</f>
+        <v>3.0800000000000001E-2</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+      <c r="Q19" s="13">
         <v>45657</v>
       </c>
-      <c r="Q19" s="13">
+      <c r="R19" s="13">
         <v>45689</v>
       </c>
-      <c r="R19" s="13">
+      <c r="S19" s="13">
         <v>45663</v>
       </c>
-      <c r="S19" s="13">
+      <c r="T19" s="13">
         <v>45690</v>
       </c>
-      <c r="T19" t="str">
-        <f t="shared" si="6"/>
+      <c r="U19" t="str">
+        <f>C19</f>
         <v>Job</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1117</v>
       </c>
@@ -6939,58 +7033,63 @@
         <v>745</v>
       </c>
       <c r="F20" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>19.102564102564102</v>
       </c>
       <c r="G20">
         <v>39</v>
       </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="10">
+      <c r="H20">
+        <v>1114</v>
+      </c>
+      <c r="I20" s="40">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="J20" s="10">
         <v>87.5</v>
       </c>
-      <c r="J20" s="17">
+      <c r="K20" s="17">
+        <f>J20/A20</f>
+        <v>7.8334825425246196E-2</v>
+      </c>
+      <c r="L20" s="9">
+        <f>A20/E20</f>
+        <v>1.4993288590604026</v>
+      </c>
+      <c r="M20" s="8">
+        <f>E20/$E$23</f>
+        <v>3.2117606483876529E-2</v>
+      </c>
+      <c r="N20">
+        <f>T20-Q20</f>
+        <v>52</v>
+      </c>
+      <c r="O20" s="11">
+        <f>ROUND(N20/E20,4)</f>
+        <v>6.9800000000000001E-2</v>
+      </c>
+      <c r="P20">
         <f t="shared" si="0"/>
-        <v>7.8334825425246196E-2</v>
-      </c>
-      <c r="K20" s="9">
-        <f t="shared" si="4"/>
-        <v>1.4993288590604026</v>
-      </c>
-      <c r="L20" s="8">
-        <f t="shared" si="5"/>
-        <v>3.2117606483876529E-2</v>
-      </c>
-      <c r="M20">
-        <f>S20-P20</f>
         <v>52</v>
       </c>
-      <c r="N20" s="11">
-        <f t="shared" si="8"/>
-        <v>6.9800000000000001E-2</v>
-      </c>
-      <c r="O20">
-        <f t="shared" si="2"/>
-        <v>52</v>
-      </c>
-      <c r="P20" s="13">
+      <c r="Q20" s="13">
         <v>45667</v>
       </c>
-      <c r="Q20" s="13">
+      <c r="R20" s="13">
         <v>45672</v>
       </c>
-      <c r="R20" s="13">
+      <c r="S20" s="13">
         <v>45669</v>
       </c>
-      <c r="S20" s="13">
+      <c r="T20" s="13">
         <v>45719</v>
       </c>
-      <c r="T20" t="str">
-        <f t="shared" si="6"/>
+      <c r="U20" t="str">
+        <f>C20</f>
         <v>The Five Scrolls</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1721</v>
       </c>
@@ -7007,52 +7106,57 @@
         <v>1042</v>
       </c>
       <c r="F21" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>29.771428571428572</v>
       </c>
       <c r="G21">
         <v>35</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="10">
+      <c r="H21">
+        <v>1719</v>
+      </c>
+      <c r="I21" s="40">
+        <v>29.3</v>
+      </c>
+      <c r="J21" s="10">
         <v>125.9</v>
       </c>
-      <c r="J21" s="17">
+      <c r="K21" s="17">
+        <f>J21/A21</f>
+        <v>7.3155142359093553E-2</v>
+      </c>
+      <c r="L21" s="9">
+        <f>A21/E21</f>
+        <v>1.6516314779270633</v>
+      </c>
+      <c r="M21" s="8">
+        <f>E21/$E$23</f>
+        <v>4.4921538196240729E-2</v>
+      </c>
+      <c r="N21">
+        <f>T21-Q21</f>
+        <v>42</v>
+      </c>
+      <c r="O21" s="11">
+        <f>ROUND(N21/E21,4)</f>
+        <v>4.0300000000000002E-2</v>
+      </c>
+      <c r="P21">
         <f t="shared" si="0"/>
-        <v>7.3155142359093553E-2</v>
-      </c>
-      <c r="K21" s="9">
-        <f t="shared" si="4"/>
-        <v>1.6516314779270633</v>
-      </c>
-      <c r="L21" s="8">
-        <f t="shared" si="5"/>
-        <v>4.4921538196240729E-2</v>
-      </c>
-      <c r="M21">
-        <f>S21-P21</f>
         <v>42</v>
       </c>
-      <c r="N21" s="11">
-        <f>ROUND(M21/E21,4)</f>
-        <v>4.0300000000000002E-2</v>
-      </c>
-      <c r="O21">
-        <f t="shared" si="2"/>
-        <v>42</v>
-      </c>
-      <c r="P21" s="13">
+      <c r="Q21" s="13">
         <v>45816</v>
       </c>
-      <c r="S21" s="13">
+      <c r="T21" s="13">
         <v>45858</v>
       </c>
-      <c r="T21" t="str">
-        <f t="shared" si="6"/>
+      <c r="U21" t="str">
+        <f>C21</f>
         <v>Daniel, Ezra, Nehemiah</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2725</v>
       </c>
@@ -7069,56 +7173,61 @@
         <v>1750</v>
       </c>
       <c r="F22" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>26.923076923076923</v>
       </c>
       <c r="G22">
         <v>65</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="10">
+      <c r="H22">
+        <v>2728</v>
+      </c>
+      <c r="I22" s="40">
+        <v>40.5</v>
+      </c>
+      <c r="J22" s="10">
         <v>195</v>
       </c>
-      <c r="J22" s="17">
-        <f t="shared" si="0"/>
+      <c r="K22" s="17">
+        <f>J22/A22</f>
         <v>7.155963302752294E-2</v>
       </c>
-      <c r="K22" s="9">
-        <f t="shared" si="4"/>
+      <c r="L22" s="9">
+        <f>A22/E22</f>
         <v>1.5571428571428572</v>
       </c>
-      <c r="L22" s="8">
-        <f t="shared" si="5"/>
+      <c r="M22" s="8">
+        <f>E22/$E$23</f>
         <v>7.5444042076220033E-2</v>
       </c>
-      <c r="M22">
-        <f t="shared" si="7"/>
+      <c r="N22">
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
-      <c r="N22" s="11">
-        <f>ROUND(M22/E22,4)</f>
+      <c r="O22" s="11">
+        <f>ROUND(N22/E22,4)</f>
         <v>1.49E-2</v>
       </c>
-      <c r="O22">
-        <f>ROUND(($N$6+$N$16)/2*E22,0)</f>
+      <c r="P22">
+        <f>ROUND(($O$6+$O$16)/2*E22,0)</f>
         <v>12</v>
       </c>
-      <c r="P22" s="13">
-        <f>S21</f>
+      <c r="Q22" s="13">
+        <f>T21</f>
         <v>45858</v>
       </c>
-      <c r="R22" s="13">
+      <c r="S22" s="13">
         <v>45869</v>
       </c>
-      <c r="S22" s="13">
+      <c r="T22" s="13">
         <v>45884</v>
       </c>
-      <c r="T22" t="str">
-        <f t="shared" si="6"/>
+      <c r="U22" t="str">
+        <f>C22</f>
         <v>Chronicles</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23">
         <f>SUM(A5:A22)</f>
         <v>34442</v>
@@ -7132,42 +7241,49 @@
         <v>23196</v>
       </c>
       <c r="F23" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>24.968783638320776</v>
       </c>
       <c r="G23">
         <f>SUM(G4:G22)</f>
         <v>929</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="16">
-        <f>SUM(I5:I22)</f>
+      <c r="H23">
+        <f>SUM(H4:H22)</f>
+        <v>34374</v>
+      </c>
+      <c r="I23">
+        <f>SUM(I4:I22)</f>
+        <v>794.4</v>
+      </c>
+      <c r="J23" s="16">
+        <f>SUM(J5:J22)</f>
         <v>2602.1000000000004</v>
       </c>
-      <c r="J23" s="17">
-        <f t="shared" si="0"/>
+      <c r="K23" s="17">
+        <f>J23/A23</f>
         <v>7.5550200336798101E-2</v>
       </c>
-      <c r="K23" s="9">
-        <f t="shared" si="4"/>
+      <c r="L23" s="9">
+        <f>A23/E23</f>
         <v>1.4848249698223832</v>
       </c>
-      <c r="P23" s="13">
-        <f>MIN(P5:P22)</f>
+      <c r="Q23" s="13">
+        <f>MIN(Q5:Q22)</f>
         <v>45657</v>
       </c>
-      <c r="S23" s="13">
-        <f>MAX(S5:S22)</f>
+      <c r="T23" s="13">
+        <f>MAX(T5:T22)</f>
         <v>45884</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="M24">
-        <f>S23-P23</f>
+        <f>T23-Q23</f>
         <v>227</v>
       </c>
       <c r="O24" s="12">
-        <f>S23-P23</f>
+        <f>T23-Q23</f>
         <v>227</v>
       </c>
       <c r="S24" s="13">
@@ -7175,7 +7291,7 @@
         <v>46005</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>86</v>
       </c>
@@ -7203,7 +7319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F26" s="8"/>
       <c r="I26" s="7" t="s">
         <v>745</v>
@@ -7222,7 +7338,7 @@
         <v>4.0925110132158586</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>142</v>
       </c>
@@ -7249,16 +7365,16 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
         <v>87</v>
       </c>
       <c r="B28" s="20">
-        <f t="shared" ref="B28:D45" si="9">B5</f>
+        <f t="shared" ref="B28:D45" si="3">B5</f>
         <v>1</v>
       </c>
       <c r="C28" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Genesis</v>
       </c>
       <c r="D28">
@@ -7287,24 +7403,24 @@
         <v>15.194464</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
         <v>87</v>
       </c>
       <c r="B29" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>2</v>
       </c>
       <c r="C29" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Exodus</v>
       </c>
       <c r="D29">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
       <c r="E29">
-        <f t="shared" ref="E29:E45" si="10">E6</f>
+        <f t="shared" ref="E29:E45" si="4">E6</f>
         <v>1213</v>
       </c>
       <c r="F29" s="20">
@@ -7313,36 +7429,36 @@
       <c r="G29" s="20"/>
       <c r="H29" s="20"/>
       <c r="I29" s="35">
-        <f t="shared" ref="I29:I45" si="11">$I$27*F29</f>
+        <f t="shared" ref="I29:I45" si="5">$I$27*F29</f>
         <v>7.12</v>
       </c>
       <c r="J29" s="35">
-        <f t="shared" ref="J29:J45" si="12">$J$27*F29</f>
+        <f t="shared" ref="J29:J45" si="6">$J$27*F29</f>
         <v>31.89404</v>
       </c>
       <c r="K29" s="35">
-        <f t="shared" ref="K29:K46" si="13">J29*$K$27</f>
+        <f t="shared" ref="K29:K46" si="7">J29*$K$27</f>
         <v>12.757616000000001</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
         <v>87</v>
       </c>
       <c r="B30" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
       <c r="C30" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Leviticus</v>
       </c>
       <c r="D30">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>27</v>
       </c>
       <c r="E30">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>859</v>
       </c>
       <c r="F30" s="20">
@@ -7351,15 +7467,15 @@
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
       <c r="I30" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>4.84</v>
       </c>
       <c r="J30" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>21.680780000000002</v>
       </c>
       <c r="K30" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>8.6723120000000016</v>
       </c>
       <c r="L30" s="20"/>
@@ -7374,28 +7490,28 @@
         <v>341</v>
       </c>
       <c r="Q30" s="1">
-        <f t="shared" ref="Q30:Q35" si="14">P30/O30</f>
+        <f t="shared" ref="Q30:Q35" si="8">P30/O30</f>
         <v>9.1298527443105751E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
         <v>87</v>
       </c>
       <c r="B31" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="C31" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Numbers</v>
       </c>
       <c r="D31">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>36</v>
       </c>
       <c r="E31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1288</v>
       </c>
       <c r="F31" s="20">
@@ -7404,15 +7520,15 @@
       <c r="G31" s="20"/>
       <c r="H31" s="20"/>
       <c r="I31" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>6.9</v>
       </c>
       <c r="J31" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>30.908550000000002</v>
       </c>
       <c r="K31" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>12.363420000000001</v>
       </c>
       <c r="L31" s="20"/>
@@ -7427,28 +7543,28 @@
         <v>1297</v>
       </c>
       <c r="Q31" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="8"/>
         <v>0.29211711711711713</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
         <v>87</v>
       </c>
       <c r="B32" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="C32" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Deuteronomy</v>
       </c>
       <c r="D32">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>34</v>
       </c>
       <c r="E32">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>959</v>
       </c>
       <c r="F32" s="20">
@@ -7462,15 +7578,15 @@
         <v>1660</v>
       </c>
       <c r="I32" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>5.86</v>
       </c>
       <c r="J32" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>26.249870000000001</v>
       </c>
       <c r="K32" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>10.499948000000002</v>
       </c>
       <c r="L32" s="20">
@@ -7488,7 +7604,7 @@
         <v>1239</v>
       </c>
       <c r="Q32" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="8"/>
         <v>9.5860735009671183E-2</v>
       </c>
     </row>
@@ -7497,19 +7613,19 @@
         <v>87</v>
       </c>
       <c r="B33" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
       <c r="C33" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Joshua, Judges</v>
       </c>
       <c r="D33">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>45</v>
       </c>
       <c r="E33">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1276</v>
       </c>
       <c r="F33" s="20">
@@ -7518,15 +7634,15 @@
       <c r="G33" s="20"/>
       <c r="H33" s="20"/>
       <c r="I33" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>7.86</v>
       </c>
       <c r="J33" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>35.208870000000005</v>
       </c>
       <c r="K33" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>14.083548000000002</v>
       </c>
       <c r="L33" s="20"/>
@@ -7541,7 +7657,7 @@
         <v>255</v>
       </c>
       <c r="Q33" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="8"/>
         <v>0.12160228898426323</v>
       </c>
     </row>
@@ -7550,19 +7666,19 @@
         <v>87</v>
       </c>
       <c r="B34" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
       <c r="C34" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Samuel</v>
       </c>
       <c r="D34">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>55</v>
       </c>
       <c r="E34">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1505</v>
       </c>
       <c r="F34" s="20">
@@ -7571,15 +7687,15 @@
       <c r="G34" s="20"/>
       <c r="H34" s="20"/>
       <c r="I34" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>9.34</v>
       </c>
       <c r="J34" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>41.838529999999999</v>
       </c>
       <c r="K34" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>16.735412</v>
       </c>
       <c r="L34" s="20"/>
@@ -7593,7 +7709,7 @@
         <v>3132</v>
       </c>
       <c r="Q34" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="8"/>
         <v>0.13501745915420096</v>
       </c>
     </row>
@@ -7602,19 +7718,19 @@
         <v>87</v>
       </c>
       <c r="B35" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
       <c r="C35" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Kings</v>
       </c>
       <c r="D35">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>47</v>
       </c>
       <c r="E35">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1536</v>
       </c>
       <c r="F35" s="20">
@@ -7623,15 +7739,15 @@
       <c r="G35" s="20"/>
       <c r="H35" s="20"/>
       <c r="I35" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>9.7000000000000011</v>
       </c>
       <c r="J35" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>43.451149999999998</v>
       </c>
       <c r="K35" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>17.380459999999999</v>
       </c>
       <c r="L35" s="20">
@@ -7651,7 +7767,7 @@
         <v>2791</v>
       </c>
       <c r="Q35" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="8"/>
         <v>0.14340766622135442</v>
       </c>
     </row>
@@ -7660,19 +7776,19 @@
         <v>87</v>
       </c>
       <c r="B36" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
       <c r="C36" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Isaiah</v>
       </c>
       <c r="D36">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>66</v>
       </c>
       <c r="E36">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1291</v>
       </c>
       <c r="F36" s="20">
@@ -7681,15 +7797,15 @@
       <c r="G36" s="20"/>
       <c r="H36" s="20"/>
       <c r="I36" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>7.54</v>
       </c>
       <c r="J36" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>33.77543</v>
       </c>
       <c r="K36" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>13.510172000000001</v>
       </c>
       <c r="L36" s="20"/>
@@ -7700,19 +7816,19 @@
         <v>87</v>
       </c>
       <c r="B37" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="C37" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Jeremiah</v>
       </c>
       <c r="D37">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>52</v>
       </c>
       <c r="E37">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1364</v>
       </c>
       <c r="F37" s="20">
@@ -7721,15 +7837,15 @@
       <c r="G37" s="20"/>
       <c r="H37" s="20"/>
       <c r="I37" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>8.52</v>
       </c>
       <c r="J37" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>38.16534</v>
       </c>
       <c r="K37" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>15.266136000000001</v>
       </c>
       <c r="L37" s="20"/>
@@ -7749,19 +7865,19 @@
         <v>87</v>
       </c>
       <c r="B38" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
       <c r="C38" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Ezekiel</v>
       </c>
       <c r="D38">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>48</v>
       </c>
       <c r="E38">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1273</v>
       </c>
       <c r="F38" s="20">
@@ -7770,15 +7886,15 @@
       <c r="G38" s="20"/>
       <c r="H38" s="20"/>
       <c r="I38" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>7.78</v>
       </c>
       <c r="J38" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>34.85051</v>
       </c>
       <c r="K38" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>13.940204000000001</v>
       </c>
       <c r="N38" t="s">
@@ -7796,19 +7912,19 @@
         <v>87</v>
       </c>
       <c r="B39" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="C39" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>The Twelve</v>
       </c>
       <c r="D39">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>67</v>
       </c>
       <c r="E39">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1050</v>
       </c>
       <c r="F39" s="20">
@@ -7822,15 +7938,15 @@
         <v>2864</v>
       </c>
       <c r="I39" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>6.54</v>
       </c>
       <c r="J39" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>29.295930000000002</v>
       </c>
       <c r="K39" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>11.718372000000002</v>
       </c>
       <c r="L39" s="20">
@@ -7844,19 +7960,19 @@
         <v>87</v>
       </c>
       <c r="B40" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="C40" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Psalms</v>
       </c>
       <c r="D40">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>150</v>
       </c>
       <c r="E40">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>2527</v>
       </c>
       <c r="F40" s="20">
@@ -7865,15 +7981,15 @@
       <c r="G40" s="20"/>
       <c r="H40" s="20"/>
       <c r="I40" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>11.700000000000001</v>
       </c>
       <c r="J40" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>52.410150000000002</v>
       </c>
       <c r="K40" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>20.964060000000003</v>
       </c>
       <c r="L40" s="20"/>
@@ -7900,19 +8016,19 @@
         <v>87</v>
       </c>
       <c r="B41" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="C41" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Proverbs</v>
       </c>
       <c r="D41">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>31</v>
       </c>
       <c r="E41">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>915</v>
       </c>
       <c r="F41" s="20">
@@ -7921,15 +8037,15 @@
       <c r="G41" s="20"/>
       <c r="H41" s="20"/>
       <c r="I41" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="J41" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>17.917999999999999</v>
       </c>
       <c r="K41" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>7.1672000000000002</v>
       </c>
       <c r="L41" s="20"/>
@@ -7956,19 +8072,19 @@
         <v>87</v>
       </c>
       <c r="B42" s="34">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
       <c r="C42" s="34" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Job</v>
       </c>
       <c r="D42" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>42</v>
       </c>
       <c r="E42" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1070</v>
       </c>
       <c r="F42" s="34">
@@ -7977,15 +8093,15 @@
       <c r="G42" s="20"/>
       <c r="H42" s="20"/>
       <c r="I42" s="37">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>5.58</v>
       </c>
       <c r="J42" s="37">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>24.995609999999999</v>
       </c>
       <c r="K42" s="37">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>9.9982439999999997</v>
       </c>
       <c r="L42" s="20">
@@ -8015,34 +8131,34 @@
         <v>87</v>
       </c>
       <c r="B43" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="C43" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>The Five Scrolls</v>
       </c>
       <c r="D43">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>39</v>
       </c>
       <c r="E43">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>745</v>
       </c>
       <c r="F43" s="20">
         <v>226</v>
       </c>
       <c r="I43" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>4.5200000000000005</v>
       </c>
       <c r="J43" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>20.247340000000001</v>
       </c>
       <c r="K43" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>8.0989360000000001</v>
       </c>
       <c r="N43" s="20" t="s">
@@ -8067,19 +8183,19 @@
         <v>87</v>
       </c>
       <c r="B44" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="C44" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Daniel, Ezra, Nehemiah</v>
       </c>
       <c r="D44">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>35</v>
       </c>
       <c r="E44">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1042</v>
       </c>
       <c r="F44" s="20">
@@ -8088,15 +8204,15 @@
       <c r="G44" s="20"/>
       <c r="H44" s="20"/>
       <c r="I44" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>6.38</v>
       </c>
       <c r="J44" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>28.57921</v>
       </c>
       <c r="K44" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>11.431684000000001</v>
       </c>
       <c r="L44" s="20"/>
@@ -8107,19 +8223,19 @@
         <v>87</v>
       </c>
       <c r="B45" s="20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>18</v>
       </c>
       <c r="C45" s="20" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>Chronicles</v>
       </c>
       <c r="D45">
-        <f t="shared" si="9"/>
+        <f t="shared" si="3"/>
         <v>65</v>
       </c>
       <c r="E45">
-        <f t="shared" si="10"/>
+        <f t="shared" si="4"/>
         <v>1750</v>
       </c>
       <c r="F45" s="20">
@@ -8133,15 +8249,15 @@
         <v>2111</v>
       </c>
       <c r="I45" s="35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="5"/>
         <v>10.040000000000001</v>
       </c>
       <c r="J45" s="35">
-        <f t="shared" si="12"/>
+        <f t="shared" si="6"/>
         <v>44.974180000000004</v>
       </c>
       <c r="K45" s="35">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>17.989672000000002</v>
       </c>
       <c r="L45" s="20">
@@ -8182,7 +8298,7 @@
         <v>594.42965000000004</v>
       </c>
       <c r="K46" s="33">
-        <f t="shared" si="13"/>
+        <f t="shared" si="7"/>
         <v>237.77186000000003</v>
       </c>
       <c r="L46" s="33">

</xml_diff>